<commit_message>
Add manufacturer SDS and TDS batch 004-006
</commit_message>
<xml_diff>
--- a/products_categories_descriptions_documents_working.xlsx
+++ b/products_categories_descriptions_documents_working.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" r:id="Rb94d85413b9248e5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" r:id="R3f1ad656eb334bb3"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -843,6 +843,12 @@
       <x:c r="W8" t="str">
         <x:v>Eggshell=https://media.benjaminmoore.com/WebServices/prod/assets/production/datasheets/TDS_0626/F626_TDS_CE.pdf|Matte=https://media.benjaminmoore.com/WebServices/prod/assets/production/datasheets/TDS_0624/F624_TDS_CE.pdf|Satin Pearl=https://media.benjaminmoore.com/WebServices/prod/assets/production/datasheets/TDS_0628/F628_TDS_CE.pdf|Semi Gloss=https://media.benjaminmoore.com/WebServices/prod/assets/production/datasheets/TDS_0627/F627_TDS_CE.pdf</x:v>
       </x:c>
+      <x:c r="X8" t="str">
+        <x:v>Eggshell=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-F6261X_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-F6262X_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-F6263X_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-F6264X_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-F62601_SDS_EN.pdf?raw=true|Matte=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-F6241X_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-F6242X_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-F6243X_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-F6244X_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-F62401_SDS_EN.pdf?raw=true|Satin Pearl=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-F6281X_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-F6282X_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-F6283X_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-F6284X_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-F62801_SDS_EN.pdf?raw=true|Semi Gloss=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-F6271X_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-F6272X_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-F6273X_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-F6274X_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-F62701_SDS_EN.pdf?raw=true</x:v>
+      </x:c>
+      <x:c r="Z8" t="str">
+        <x:v>Eggshell=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/benjamin-moore-F626_TDS_CE.pdf?raw=true|Matte=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/benjamin-moore-F624_TDS_CE.pdf?raw=true|Satin Pearl=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/benjamin-moore-F628_TDS_CE.pdf?raw=true|Semi Gloss=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/benjamin-moore-F627_TDS_CE.pdf?raw=true</x:v>
+      </x:c>
     </x:row>
     <x:row r="9">
       <x:c r="A9" t="str">
@@ -904,6 +910,12 @@
       <x:c r="W9" t="str">
         <x:v>Pearl=https://media.benjaminmoore.com/WebServices/prod/assets/production/datasheets/TDS_0322/Y322_TDS_CE.pdf</x:v>
       </x:c>
+      <x:c r="X9" t="str">
+        <x:v>Pearl=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-F32201_MSDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-F3221B_MSDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-F3222B_MSDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-F3223B_MSDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-F3224B_MSDS_EN.pdf?raw=true</x:v>
+      </x:c>
+      <x:c r="Z9" t="str">
+        <x:v>Pearl=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/benjamin-moore-Y322_TDS_CE.pdf?raw=true</x:v>
+      </x:c>
     </x:row>
     <x:row r="10">
       <x:c r="A10" t="str">
@@ -964,6 +976,12 @@
       </x:c>
       <x:c r="W10" t="str">
         <x:v>Ultra Flat=https://media.benjaminmoore.com/WebServices/prod/assets/production/datasheets/TDS_0508/F508_TDS_CE.pdf</x:v>
+      </x:c>
+      <x:c r="X10" t="str">
+        <x:v>Ultra Flat=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-F50809_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-F5081X_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-F5082X_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-F5083X_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-F5084X_SDS_EN.pdf?raw=true</x:v>
+      </x:c>
+      <x:c r="Z10" t="str">
+        <x:v>Ultra Flat=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/benjamin-moore-F508_TDS_CE.pdf?raw=true</x:v>
       </x:c>
     </x:row>
     <x:row r="11">

</xml_diff>

<commit_message>
Add manufacturer SDS and TDS batch 007-009
</commit_message>
<xml_diff>
--- a/products_categories_descriptions_documents_working.xlsx
+++ b/products_categories_descriptions_documents_working.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" r:id="R3f1ad656eb334bb3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" r:id="Rf6e2810288e64ea5"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1044,6 +1044,12 @@
       <x:c r="W11" t="str">
         <x:v>Flat=https://media.benjaminmoore.com/WebServices/prod/assets/production/datasheets/TDS_0258/258_TDS_CE.pdf</x:v>
       </x:c>
+      <x:c r="X11" t="str">
+        <x:v>Flat=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-K25801_SDS_EN.pdf?raw=true</x:v>
+      </x:c>
+      <x:c r="Z11" t="str">
+        <x:v>Flat=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/benjamin-moore-258_TDS_CE.pdf?raw=true</x:v>
+      </x:c>
     </x:row>
     <x:row r="12">
       <x:c r="A12" t="str">
@@ -1105,6 +1111,12 @@
       <x:c r="W12" t="str">
         <x:v>Flat=https://media.benjaminmoore.com/WebServices/prod/assets/production/datasheets/TDS_0629/F629_TDS_CE.pdf|Satin=https://media.benjaminmoore.com/WebServices/prod/assets/production/datasheets/TDS_0631/F631_TDS_CE.pdf|Soft Gloss=https://media.benjaminmoore.com/WebServices/prod/assets/production/datasheets/TDS_0632/F632_TDS_CE.pdf|Low Lustre=https://media.benjaminmoore.com/WebServices/prod/assets/production/datasheets/TDS_0634/F634_TDS_CE.pdf</x:v>
       </x:c>
+      <x:c r="X12" t="str">
+        <x:v>Flat=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-F6291X_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-F6292X_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-F6293X_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-F6294X_SDS_EN.pdf?raw=true|Low Lustre=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-F6341X_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-F6342X_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-F6343X_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-F6344X_SDS_EN.pdf?raw=true|Satin=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-F6311X_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-F6312X_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-F6313X_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-F6314X_SDS_EN.pdf?raw=true</x:v>
+      </x:c>
+      <x:c r="Z12" t="str">
+        <x:v>Flat=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/benjamin-moore-F629_TDS_CE.pdf?raw=true|Satin=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/benjamin-moore-F631_TDS_CE.pdf?raw=true|Soft Gloss=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/benjamin-moore-F632_TDS_CE.pdf?raw=true|Low Lustre=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/benjamin-moore-F634_TDS_CE.pdf?raw=true</x:v>
+      </x:c>
     </x:row>
     <x:row r="13">
       <x:c r="A13" t="str">
@@ -1165,6 +1177,12 @@
       </x:c>
       <x:c r="W13" t="str">
         <x:v>Flat=https://media.benjaminmoore.com/WebServices/prod/assets/production/datasheets/TDS_0400/K400_TDS_CE.pdf|Low Lustre=https://media.benjaminmoore.com/WebServices/prod/assets/production/datasheets/TDS_0401/K401_TDS_CE.pdf|Soft Gloss=https://media.benjaminmoore.com/WebServices/prod/assets/production/datasheets/TDS_0403/F403_TDS_CE.pdf</x:v>
+      </x:c>
+      <x:c r="X13" t="str">
+        <x:v>Flat=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-K40001_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-K4001X_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-K4002X_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-K4003X_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-K4004X_SDS_EN.pdf?raw=true|Low Lustre=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-K40101_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-K4011X_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-K4012X_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-K4013X_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-K4014X_SDS_EN.pdf?raw=true|Soft Gloss=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-F40380_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-F40301_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-F4031X_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-F4032X_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-F4033X_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-F4034X_SDS_EN.pdf?raw=true</x:v>
+      </x:c>
+      <x:c r="Z13" t="str">
+        <x:v>Flat=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/benjamin-moore-K400_TDS_CE.pdf?raw=true|Low Lustre=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/benjamin-moore-K401_TDS_CE.pdf?raw=true|Soft Gloss=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/benjamin-moore-F403_TDS_CE.pdf?raw=true</x:v>
       </x:c>
     </x:row>
     <x:row r="14">

</xml_diff>

<commit_message>
Add manufacturer SDS and TDS batch 010-012
</commit_message>
<xml_diff>
--- a/products_categories_descriptions_documents_working.xlsx
+++ b/products_categories_descriptions_documents_working.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" r:id="Rf6e2810288e64ea5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" r:id="R55f40c228feb457e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1245,6 +1245,12 @@
       <x:c r="W14" t="str">
         <x:v>Flat=https://media.benjaminmoore.com/WebServices/prod/assets/production/datasheets/TDS_0763/K763_TDS_CE.pdf|Low Lustre=https://media.benjaminmoore.com/WebServices/prod/assets/production/datasheets/TDS_0764/K764_TDS_CE.pdf|Soft Gloss=https://media.benjaminmoore.com/WebServices/prod/assets/production/datasheets/TDS_0765/K765_TDS_CE.pdf</x:v>
       </x:c>
+      <x:c r="X14" t="str">
+        <x:v>Flat=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-K7631X_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-K7632X_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-K7633X_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-K7634X_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-K76301_SDS_EN.pdf?raw=true|Low Lustre=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-K7641X_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-K7642X_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-K7643X_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-K7644X_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-K76401_SDS_EN.pdf?raw=true|Soft Gloss=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-K7651X_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-K7652X_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-K7653X_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-K7654X_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-K76501_SDS_EN.pdf?raw=true</x:v>
+      </x:c>
+      <x:c r="Z14" t="str">
+        <x:v>Flat=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/benjamin-moore-K763_TDS_CE.pdf?raw=true|Low Lustre=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/benjamin-moore-K764_TDS_CE.pdf?raw=true|Soft Gloss=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/benjamin-moore-K765_TDS_CE.pdf?raw=true</x:v>
+      </x:c>
     </x:row>
     <x:row r="15">
       <x:c r="A15" t="str">
@@ -1306,6 +1312,12 @@
       <x:c r="W15" t="str">
         <x:v>Flat=https://media.benjaminmoore.com/WebServices/prod/assets/production/datasheets/TDS_0447/Y447_TDS_CE.pdf|Low Lustre=https://media.benjaminmoore.com/WebServices/prod/assets/production/datasheets/TDS_0455/Y455_TDS_CE.pdf|Satin=https://media.benjaminmoore.com/WebServices/prod/assets/production/datasheets/TDS_0448/Y448_TDS_CE.pdf|Soft Gloss=https://media.benjaminmoore.com/WebServices/prod/assets/production/datasheets/TDS_0449/Y449_TDS_CE.pdf</x:v>
       </x:c>
+      <x:c r="X15" t="str">
+        <x:v>Flat=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-Y4471X_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-Y4472X_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-Y4473X_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-Y4474X_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-Y44701_SDS_EN.pdf?raw=true|Low Lustre=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-Y4551X_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-Y4552X_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-Y4553X_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-Y4554X_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-Y45501_SDS_EN.pdf?raw=true|Satin=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-Y4481X_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-Y4482X_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-Y4483X_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-Y4484X_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-Y44801_SDS_EN.pdf?raw=true|Soft Gloss=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-Y4491X_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-Y4492X_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-Y4493X_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-Y4494X_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-Y44901_SDS_EN.pdf?raw=true</x:v>
+      </x:c>
+      <x:c r="Z15" t="str">
+        <x:v>Flat=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/benjamin-moore-Y447_TDS_CE.pdf?raw=true|Low Lustre=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/benjamin-moore-Y455_TDS_CE.pdf?raw=true|Satin=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/benjamin-moore-Y448_TDS_CE.pdf?raw=true|Soft Gloss=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/benjamin-moore-Y449_TDS_CE.pdf?raw=true</x:v>
+      </x:c>
     </x:row>
     <x:row r="16">
       <x:c r="A16" t="str">
@@ -1366,6 +1378,12 @@
       </x:c>
       <x:c r="W16" t="str">
         <x:v>Semi Solid=https://media.benjaminmoore.com/WebServices/prod/assets/production/datasheets/TDS_0693/K693_TDS_CE.pdf|Semi Transparent=https://media.benjaminmoore.com/WebServices/prod/assets/production/datasheets/TDS_0692/K692_TDS_CE.pdf|Translucent=https://media.benjaminmoore.com/WebServices/prod/assets/production/datasheets/TDS_0691/K691_TDS_CE.pdf</x:v>
+      </x:c>
+      <x:c r="X16" t="str">
+        <x:v>Semi Solid=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-K69301_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-K69306_SDS_EN.pdf?raw=true|Semi Transparent=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-K69206_SDS_EN.pdf?raw=true|Translucent=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-K69178_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-K69140_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-K69165_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-K69160_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-K69110_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-K69120_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-K69130_SDS_EN.pdf?raw=true</x:v>
+      </x:c>
+      <x:c r="Z16" t="str">
+        <x:v>Semi Solid=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/benjamin-moore-K693_TDS_CE.pdf?raw=true|Semi Transparent=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/benjamin-moore-K692_TDS_CE.pdf?raw=true|Translucent=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/benjamin-moore-K691_TDS_CE.pdf?raw=true</x:v>
       </x:c>
     </x:row>
     <x:row r="17">

</xml_diff>

<commit_message>
Add manufacturer SDS and TDS batch 013-015
</commit_message>
<xml_diff>
--- a/products_categories_descriptions_documents_working.xlsx
+++ b/products_categories_descriptions_documents_working.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" r:id="R55f40c228feb457e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" r:id="Rf723825c07d043e3"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1444,6 +1444,12 @@
       <x:c r="W17" t="str">
         <x:v>Semi Solid=https://media.benjaminmoore.com/WebServices/prod/assets/production/datasheets/TDS_0593/K593_TDS_CE.pdf|Semi Transparent=https://media.benjaminmoore.com/WebServices/prod/assets/production/datasheets/TDS_0592/K592_TDS_CE.pdf|Translucent=https://media.benjaminmoore.com/WebServices/prod/assets/production/datasheets/TDS_0591/K591_TDS_CE.pdf</x:v>
       </x:c>
+      <x:c r="X17" t="str">
+        <x:v>Semi Solid=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-K59306_SDS_EN.pdf?raw=true|Semi Transparent=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-K59206_SDS_EN.pdf?raw=true|Translucent=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-K59178_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-K59140_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-K59165_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-K59160_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-K59110_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-K59120_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-K59130_SDS_EN.pdf?raw=true</x:v>
+      </x:c>
+      <x:c r="Z17" t="str">
+        <x:v>Semi Solid=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/benjamin-moore-K593_TDS_CE.pdf?raw=true|Semi Transparent=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/benjamin-moore-K592_TDS_CE.pdf?raw=true|Translucent=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/benjamin-moore-K591_TDS_CE.pdf?raw=true</x:v>
+      </x:c>
     </x:row>
     <x:row r="18">
       <x:c r="A18" t="str">
@@ -1505,6 +1511,12 @@
       <x:c r="W18" t="str">
         <x:v>Solid=https://media.benjaminmoore.com/WebServices/prod/assets/production/datasheets/TDS_0694/K694_TDS_CE.pdf|Semi Solid=https://media.benjaminmoore.com/WebServices/prod/assets/production/datasheets/TDS_0693/K693_TDS_CE.pdf|Semi Transparent=https://media.benjaminmoore.com/WebServices/prod/assets/production/datasheets/TDS_0692/K692_TDS_CE.pdf|Translucent=https://media.benjaminmoore.com/WebServices/prod/assets/production/datasheets/TDS_0691/K691_TDS_CE.pdf</x:v>
       </x:c>
+      <x:c r="X18" t="str">
+        <x:v>Solid=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-K6941X_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-K6942X_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-K6943X_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-K6944X_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-K69401_SDS_EN.pdf?raw=true</x:v>
+      </x:c>
+      <x:c r="Z18" t="str">
+        <x:v>Solid=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/benjamin-moore-K694_TDS_CE.pdf?raw=true|Semi Solid=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/benjamin-moore-K693_TDS_CE.pdf?raw=true|Semi Transparent=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/benjamin-moore-K692_TDS_CE.pdf?raw=true|Translucent=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/benjamin-moore-K691_TDS_CE.pdf?raw=true</x:v>
+      </x:c>
     </x:row>
     <x:row r="19">
       <x:c r="A19" t="str">
@@ -1563,6 +1575,12 @@
       </x:c>
       <x:c r="W19" t="str">
         <x:v>Primer=https://media.benjaminmoore.com/WebServices/prod/assets/production/datasheets/TDS_0046/K046_TDS_CE.pdf</x:v>
+      </x:c>
+      <x:c r="X19" t="str">
+        <x:v>Primer=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-K04600_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-K04604_SDS_EN.pdf?raw=true</x:v>
+      </x:c>
+      <x:c r="Z19" t="str">
+        <x:v>Primer=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/benjamin-moore-K046_TDS_CE.pdf?raw=true</x:v>
       </x:c>
     </x:row>
     <x:row r="20">

</xml_diff>

<commit_message>
Add manufacturer SDS and TDS batch 016-018
</commit_message>
<xml_diff>
--- a/products_categories_descriptions_documents_working.xlsx
+++ b/products_categories_descriptions_documents_working.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" r:id="Rf723825c07d043e3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" r:id="R3b2f4daa25074707"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1641,6 +1641,12 @@
       <x:c r="W20" t="str">
         <x:v>Primer=https://media.benjaminmoore.com/WebServices/prod/assets/production/datasheets/TDS_SXA-110/SXA110_TDS_CE.pdf</x:v>
       </x:c>
+      <x:c r="X20" t="str">
+        <x:v>Primer=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/insl-x-SXA-1100F_SDS_EN.pdf?raw=true</x:v>
+      </x:c>
+      <x:c r="Z20" t="str">
+        <x:v>Primer=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/insl-x-SXA110_TDS_CE.pdf?raw=true</x:v>
+      </x:c>
     </x:row>
     <x:row r="21">
       <x:c r="A21" t="str">
@@ -1700,6 +1706,12 @@
       <x:c r="W21" t="str">
         <x:v>Primer=https://media.benjaminmoore.com/WebServices/prod/assets/production/datasheets/TDS_507/K507_TDS_CE.pdf</x:v>
       </x:c>
+      <x:c r="X21" t="str">
+        <x:v>Primer=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-K50700_SDS_EN.pdf?raw=true</x:v>
+      </x:c>
+      <x:c r="Z21" t="str">
+        <x:v>Primer=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/benjamin-moore-K507_TDS_CE.pdf?raw=true</x:v>
+      </x:c>
     </x:row>
     <x:row r="22">
       <x:c r="A22" t="str">
@@ -1758,6 +1770,12 @@
       </x:c>
       <x:c r="W22" t="str">
         <x:v>Primer=https://media.benjaminmoore.com/WebServices/prod/assets/production/datasheets/TDS_0265/K265_TDS_CE.pdf</x:v>
+      </x:c>
+      <x:c r="X22" t="str">
+        <x:v>Primer=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-K26500_SDS_EN.pdf?raw=true</x:v>
+      </x:c>
+      <x:c r="Z22" t="str">
+        <x:v>Primer=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/benjamin-moore-K265_TDS_CE.pdf?raw=true</x:v>
       </x:c>
     </x:row>
     <x:row r="23">

</xml_diff>

<commit_message>
Add manufacturer SDS and TDS batch 019-021
</commit_message>
<xml_diff>
--- a/products_categories_descriptions_documents_working.xlsx
+++ b/products_categories_descriptions_documents_working.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" r:id="R3b2f4daa25074707"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" r:id="Re311f305d2a7462e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1838,6 +1838,12 @@
       <x:c r="W23" t="str">
         <x:v>High Gloss=https://media.benjaminmoore.com/WebServices/prod/assets/production/datasheets/TDS_0794/F794_TDS_CE.pdf|Satin=https://media.benjaminmoore.com/WebServices/prod/assets/production/datasheets/TDS_0792/K792_TDS_CE.pdf|Semi Gloss=https://media.benjaminmoore.com/WebServices/prod/assets/production/datasheets/TDS_0793/K793_TDS_CE.pdf</x:v>
       </x:c>
+      <x:c r="X23" t="str">
+        <x:v>High Gloss=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-K79401_MSDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-K7941X_MSDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-K7942X_MSDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-K7943X_MSDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-K7944X_MSDS_EN.pdf?raw=true|Satin=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-K79201_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-K7921X_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-K7922X_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-K7923X_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-K7924X_SDS_EN.pdf?raw=true|Semi Gloss=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-K79301_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-K7931X_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-K7932X_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-K7933X_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-K7934X_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-K79380_SDS_EN.pdf?raw=true</x:v>
+      </x:c>
+      <x:c r="Z23" t="str">
+        <x:v>High Gloss=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/benjamin-moore-F794_TDS_CE.pdf?raw=true|Satin=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/benjamin-moore-K792_TDS_CE.pdf?raw=true|Semi Gloss=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/benjamin-moore-K793_TDS_CE.pdf?raw=true</x:v>
+      </x:c>
     </x:row>
     <x:row r="24">
       <x:c r="A24" t="str">
@@ -1899,6 +1905,12 @@
       <x:c r="W24" t="str">
         <x:v>High Gloss=https://media.benjaminmoore.com/WebServices/prod/assets/production/datasheets/TDS_0121/K121_TDS_CE.pdf|Low Sheen=https://media.benjaminmoore.com/WebServices/prod/assets/production/datasheets/TDS_0122/F122_TDS_CE.pdf</x:v>
       </x:c>
+      <x:c r="X24" t="str">
+        <x:v>Low Sheen=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-F12201_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-F1221X_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-F1222X_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-F1223X_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-F1224X_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-F12274_SDS_EN.pdf?raw=true|High Gloss=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-K1211X_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-K1212X_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-K1213X_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-K1214X_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-K12101_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-K12174_SDS_EN.pdf?raw=true</x:v>
+      </x:c>
+      <x:c r="Z24" t="str">
+        <x:v>High Gloss=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/benjamin-moore-K121_TDS_CE.pdf?raw=true|Low Sheen=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/benjamin-moore-F122_TDS_CE.pdf?raw=true</x:v>
+      </x:c>
     </x:row>
     <x:row r="25">
       <x:c r="A25" t="str">
@@ -1959,6 +1971,12 @@
       </x:c>
       <x:c r="W25" t="str">
         <x:v>Satin=https://media.benjaminmoore.com/WebServices/prod/assets/production/datasheets/TDS_CC-65XX/CC-65XX_TDS_CE.pdf</x:v>
+      </x:c>
+      <x:c r="X25" t="str">
+        <x:v>Satin=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/insl-x-CC651BF_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/insl-x-CC652BF_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/insl-x-CC653BF_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/insl-x-CC654BF_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/insl-x-CC6501F_SDS_EN.pdf?raw=true</x:v>
+      </x:c>
+      <x:c r="Z25" t="str">
+        <x:v>Satin=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/insl-x-CC-65XX_TDS_CE.pdf?raw=true</x:v>
       </x:c>
     </x:row>
     <x:row r="26">

</xml_diff>

<commit_message>
Add manufacturer SDS and TDS batch 022-024
</commit_message>
<xml_diff>
--- a/products_categories_descriptions_documents_working.xlsx
+++ b/products_categories_descriptions_documents_working.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" r:id="Re311f305d2a7462e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" r:id="R806e53d8e13d4d2e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2039,6 +2039,12 @@
       <x:c r="W26" t="str">
         <x:v>Eggshell=https://media.benjaminmoore.com/WebServices/prod/assets/production/datasheets/TDS_0538/F538_TDS_CE.pdf|Flat=https://media.benjaminmoore.com/WebServices/prod/assets/production/datasheets/TDS_0535/F535_TDS_CE.pdf|Low Sheen Eggshell=https://media.benjaminmoore.com/WebServices/prod/assets/production/datasheets/TDS_0537/F537_TDS_CE.pdf|Satin Pearl=https://media.benjaminmoore.com/WebServices/prod/assets/production/datasheets/TDS_0545/F545_TDS_CE.pdf|Semi Gloss=https://media.benjaminmoore.com/WebServices/prod/assets/production/datasheets/TDS_0546/F546_TDS_CE.pdf</x:v>
       </x:c>
+      <x:c r="X26" t="str">
+        <x:v>Eggshell=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-F5381X_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-F5382X_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-F5383X_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-F5384X_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-F53801_SDS_EN.pdf?raw=true|Low Sheen Eggshell=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-F5371X_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-F5372X_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-F5373X_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-F5374X_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-F53701_SDS_EN.pdf?raw=true|Flat=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-F5351X_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-F5352X_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-F5353X_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-F5354X_SDS_EN.pdf?raw=true|Satin Pearl=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-F5451X_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-S5451X_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-F5452X_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-S5452X_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-F5453X_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-S5453X_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-F5454X_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-S5454X_SDS_EN.pdf?raw=true|Semi Gloss=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-K5391X_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-K5392X_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-K5393X_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-K5394X_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-F54601_SDS_EN.pdf?raw=true</x:v>
+      </x:c>
+      <x:c r="Z26" t="str">
+        <x:v>Eggshell=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/benjamin-moore-F538_TDS_CE.pdf?raw=true|Flat=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/benjamin-moore-F535_TDS_CE.pdf?raw=true|Low Sheen Eggshell=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/benjamin-moore-F537_TDS_CE.pdf?raw=true|Satin Pearl=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/benjamin-moore-F545_TDS_CE.pdf?raw=true|Semi Gloss=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/benjamin-moore-F546_TDS_CE.pdf?raw=true</x:v>
+      </x:c>
     </x:row>
     <x:row r="27">
       <x:c r="A27" t="str">
@@ -2100,6 +2106,12 @@
       <x:c r="W27" t="str">
         <x:v>Eggshell=https://media.benjaminmoore.com/WebServices/prod/assets/production/datasheets/TDS_0485/F485_TDS_CE.pdf|Matte=https://media.benjaminmoore.com/WebServices/prod/assets/production/datasheets/TDS_0484/F484_TDS_CE.pdf|Pearl=https://media.benjaminmoore.com/WebServices/prod/assets/production/datasheets/TDS_0486/F486_TDS_CE.pdf|Semi Gloss=https://media.benjaminmoore.com/WebServices/prod/assets/production/datasheets/TDS_0487/F487_TDS_CE.pdf</x:v>
       </x:c>
+      <x:c r="X27" t="str">
+        <x:v>Eggshell=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-F4851X_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-F4852X_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-F4853X_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-F4854X_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-F48501_SDS_EN.pdf?raw=true|Matte=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-F4841X_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-F4842X_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-F4843X_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-F4844X_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-F48401_SDS_EN.pdf?raw=true|Pearl=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-F4861X_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-F4862X_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-F4863X_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-F4864X_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-F48601_SDS_EN.pdf?raw=true|Semi Gloss=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-F4871X_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-F4872X_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-F4873X_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-F4874X_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-F48701_SDS_EN.pdf?raw=true</x:v>
+      </x:c>
+      <x:c r="Z27" t="str">
+        <x:v>Eggshell=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/benjamin-moore-F485_TDS_CE.pdf?raw=true|Matte=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/benjamin-moore-F484_TDS_CE.pdf?raw=true|Pearl=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/benjamin-moore-F486_TDS_CE.pdf?raw=true|Semi Gloss=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/benjamin-moore-F487_TDS_CE.pdf?raw=true</x:v>
+      </x:c>
     </x:row>
     <x:row r="28">
       <x:c r="A28" t="str">
@@ -2160,6 +2172,12 @@
       </x:c>
       <x:c r="W28" t="str">
         <x:v>Eggshell=https://media.benjaminmoore.com/WebServices/prod/assets/production/datasheets/TDS_0374/Y374_TDS_CE.pdf|Flat=https://media.benjaminmoore.com/WebServices/prod/assets/production/datasheets/TDS_0373/Y373_TDS_CE.pdf|Pearl=https://media.benjaminmoore.com/WebServices/prod/assets/production/datasheets/TDS_0375/Y375_TDS_CE.pdf|Semi Gloss=https://media.benjaminmoore.com/WebServices/prod/assets/production/datasheets/TDS_0376/Y376_TDS_CE.pdf</x:v>
+      </x:c>
+      <x:c r="X28" t="str">
+        <x:v>Eggshell=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-Y37401_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-Y3741X_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-Y3742X_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-Y3743X_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-Y3744X_SDS_EN.pdf?raw=true|Flat=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-Y37301_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-Y3731X_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-Y3732X_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-Y3733X_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-Y3734X_SDS_EN.pdf?raw=true|Pearl=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-Y37501_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-Y3751X_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-Y3752X_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-Y3753X_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-Y3754X_SDS_EN.pdf?raw=true|Semi Gloss=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-Y37601_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-Y3761X_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-Y3762X_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-Y3763X_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-Y3764X_SDS_EN.pdf?raw=true</x:v>
+      </x:c>
+      <x:c r="Z28" t="str">
+        <x:v>Eggshell=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/benjamin-moore-Y374_TDS_CE.pdf?raw=true|Flat=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/benjamin-moore-Y373_TDS_CE.pdf?raw=true|Pearl=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/benjamin-moore-Y375_TDS_CE.pdf?raw=true|Semi Gloss=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/benjamin-moore-Y376_TDS_CE.pdf?raw=true</x:v>
       </x:c>
     </x:row>
     <x:row r="29">

</xml_diff>

<commit_message>
Add manufacturer SDS and TDS batch 025-027
</commit_message>
<xml_diff>
--- a/products_categories_descriptions_documents_working.xlsx
+++ b/products_categories_descriptions_documents_working.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" r:id="R806e53d8e13d4d2e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" r:id="Rbc1158fe38344cfe"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2238,6 +2238,12 @@
       <x:c r="W29" t="str">
         <x:v>Primer=https://media.benjaminmoore.com/WebServices/prod/assets/production/datasheets/TDS_AP-1000/AP-1000_TDS_CAE.pdf</x:v>
       </x:c>
+      <x:c r="X29" t="str">
+        <x:v>Primer=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/insl-x-AP1000F_SDS_EN.pdf?raw=true</x:v>
+      </x:c>
+      <x:c r="Z29" t="str">
+        <x:v>Primer=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/insl-x-AP-1000_TDS_CAE.pdf?raw=true</x:v>
+      </x:c>
     </x:row>
     <x:row r="30">
       <x:c r="A30" t="str">
@@ -2297,6 +2303,12 @@
       <x:c r="W30" t="str">
         <x:v>Primer=https://media.benjaminmoore.com/WebServices/prod/assets/production/datasheets/TDS_AQ-0XXX/AQ-0XXX_TDS_CE.pdf</x:v>
       </x:c>
+      <x:c r="X30" t="str">
+        <x:v>Primer=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/insl-x-AQ-0400F_SDS_EN.pdf?raw=true</x:v>
+      </x:c>
+      <x:c r="Z30" t="str">
+        <x:v>Primer=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/insl-x-AQ-0XXX_TDS_CE.pdf?raw=true</x:v>
+      </x:c>
     </x:row>
     <x:row r="31">
       <x:c r="A31" t="str">
@@ -2355,6 +2367,12 @@
       </x:c>
       <x:c r="W31" t="str">
         <x:v>Primer=https://media.benjaminmoore.com/WebServices/prod/assets/production/datasheets/TDS_PS-8100/PS-8100_TDS_CE.pdf</x:v>
+      </x:c>
+      <x:c r="X31" t="str">
+        <x:v>Primer=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/insl-x-PS-8100F_SDS_EN.pdf?raw=true</x:v>
+      </x:c>
+      <x:c r="Z31" t="str">
+        <x:v>Primer=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/insl-x-PS-8100_TDS_CE.pdf?raw=true</x:v>
       </x:c>
     </x:row>
     <x:row r="32">

</xml_diff>

<commit_message>
Add manufacturer SDS and TDS batch 028-030
</commit_message>
<xml_diff>
--- a/products_categories_descriptions_documents_working.xlsx
+++ b/products_categories_descriptions_documents_working.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" r:id="Rbc1158fe38344cfe"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" r:id="R729036ab88b24e9b"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2433,6 +2433,12 @@
       <x:c r="W32" t="str">
         <x:v>Primer=https://media.benjaminmoore.com/WebServices/prod/assets/production/datasheets/TDS_SXA-110/SXA110_TDS_CE.pdf</x:v>
       </x:c>
+      <x:c r="X32" t="str">
+        <x:v>Primer=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/insl-x-SXA-1100F_SDS_EN.pdf?raw=true</x:v>
+      </x:c>
+      <x:c r="Z32" t="str">
+        <x:v>Primer=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/insl-x-SXA110_TDS_CE.pdf?raw=true</x:v>
+      </x:c>
     </x:row>
     <x:row r="33">
       <x:c r="A33" t="str">
@@ -2492,6 +2498,12 @@
       <x:c r="W33" t="str">
         <x:v>Primer=https://media.benjaminmoore.com/WebServices/prod/assets/production/datasheets/TDS_SB-5000/SB-5000_TDS_CE.pdf</x:v>
       </x:c>
+      <x:c r="X33" t="str">
+        <x:v>Primer=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/insl-x-SB-5000FR_SDS_EN.pdf?raw=true</x:v>
+      </x:c>
+      <x:c r="Z33" t="str">
+        <x:v>Primer=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/insl-x-SB-5000_TDS_CE.pdf?raw=true</x:v>
+      </x:c>
     </x:row>
     <x:row r="34">
       <x:c r="A34" t="str">
@@ -2550,6 +2562,12 @@
       </x:c>
       <x:c r="W34" t="str">
         <x:v>Primer=https://media.benjaminmoore.com/WebServices/prod/assets/production/datasheets/TDS_HB-2100/HB-2100_TDS_CAE.pdf</x:v>
+      </x:c>
+      <x:c r="X34" t="str">
+        <x:v>Primer=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/insl-x-HB2100FR_SDS_EN.pdf?raw=true</x:v>
+      </x:c>
+      <x:c r="Z34" t="str">
+        <x:v>Primer=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/insl-x-HB-2100_TDS_CAE.pdf?raw=true</x:v>
       </x:c>
     </x:row>
     <x:row r="35">

</xml_diff>

<commit_message>
Add manufacturer SDS and TDS batch 031-033
</commit_message>
<xml_diff>
--- a/products_categories_descriptions_documents_working.xlsx
+++ b/products_categories_descriptions_documents_working.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" r:id="R729036ab88b24e9b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" r:id="R6b87a1dc8eb24379"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2628,6 +2628,12 @@
       <x:c r="W35" t="str">
         <x:v>Primer=https://media.benjaminmoore.com/WebServices/prod/assets/production/datasheets/TDS_RO3000/RO-3000_TDS_CE.pdf</x:v>
       </x:c>
+      <x:c r="X35" t="str">
+        <x:v>Primer=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/insl-x-RO3000F_SDS_EN.pdf?raw=true</x:v>
+      </x:c>
+      <x:c r="Z35" t="str">
+        <x:v>Primer=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/insl-x-RO-3000_TDS_CE.pdf?raw=true</x:v>
+      </x:c>
     </x:row>
     <x:row r="36">
       <x:c r="A36" t="str">
@@ -2687,6 +2693,12 @@
       <x:c r="W36" t="str">
         <x:v>Primer=https://media.benjaminmoore.com/WebServices/prod/assets/production/datasheets/TDS_VB-5000/VB-5000_TDS_CAE.pdf</x:v>
       </x:c>
+      <x:c r="X36" t="str">
+        <x:v>Primer=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/insl-x-VB-5000F_SDS_EN.pdf?raw=true</x:v>
+      </x:c>
+      <x:c r="Z36" t="str">
+        <x:v>Primer=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/insl-x-VB-5000_TDS_CAE.pdf?raw=true</x:v>
+      </x:c>
     </x:row>
     <x:row r="37">
       <x:c r="A37" t="str">
@@ -3634,6 +3646,12 @@
       </x:c>
       <x:c r="W52" t="str">
         <x:v>Satin=https://media.benjaminmoore.com/WebServices/prod/assets/production/datasheets/TDS_CST-2XXX/CST-2XXX_TDS_CAE.pdf</x:v>
+      </x:c>
+      <x:c r="X52" t="str">
+        <x:v>Satin=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/insl-x-CST-2100F_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/insl-x-CST-2308F_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/insl-x-CST-2310F_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/insl-x-CST-2789F_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/insl-x-CST-2110F_SDS_EN.pdf?raw=true</x:v>
+      </x:c>
+      <x:c r="Z52" t="str">
+        <x:v>Satin=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/insl-x-CST-2XXX_TDS_CAE.pdf?raw=true</x:v>
       </x:c>
     </x:row>
     <x:row r="53">

</xml_diff>

<commit_message>
Add manufacturer SDS and TDS batch 034-036
</commit_message>
<xml_diff>
--- a/products_categories_descriptions_documents_working.xlsx
+++ b/products_categories_descriptions_documents_working.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" r:id="R6b87a1dc8eb24379"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" r:id="Re01872e8fd1547f3"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -3714,6 +3714,12 @@
       <x:c r="W53" t="str">
         <x:v>Semi Gloss=https://media.benjaminmoore.com/WebServices/prod/assets/production/datasheets/TDS_EGG-XXXX/EGG_XXXX_TDS_CAE.pdf</x:v>
       </x:c>
+      <x:c r="X53" t="str">
+        <x:v>Semi Gloss=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/insl-x-EGG190S9F_EN_SDS.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/insl-x-EGG310SF_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/insl-x-EGG-111F_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/insl-x-EGG10BS9F_SDS_EN.pdf?raw=true</x:v>
+      </x:c>
+      <x:c r="Z53" t="str">
+        <x:v>Semi Gloss=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/insl-x-EGG_XXXX_TDS_CAE.pdf?raw=true</x:v>
+      </x:c>
     </x:row>
     <x:row r="54">
       <x:c r="A54" t="str">
@@ -3775,6 +3781,12 @@
       <x:c r="W54" t="str">
         <x:v>Satin=https://media.benjaminmoore.com/WebServices/prod/assets/production/datasheets/TDS_CG-3XXX/CG-3XXX_TDS_CE.pdf</x:v>
       </x:c>
+      <x:c r="X54" t="str">
+        <x:v>Satin=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/insl-x-CG-301BFGHS_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/insl-x-CG-304BFGHS_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/insl-x-CG-3022FGHS_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/insl-x-CG-3007FGHS_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/insl-x-CG-3011FGHS_SDS_EN.pdf?raw=true</x:v>
+      </x:c>
+      <x:c r="Z54" t="str">
+        <x:v>Satin=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/insl-x-CG-3XXX_TDS_CE.pdf?raw=true</x:v>
+      </x:c>
     </x:row>
     <x:row r="55">
       <x:c r="A55" t="str">
@@ -3835,6 +3847,12 @@
       </x:c>
       <x:c r="W55" t="str">
         <x:v>Flat=https://media.benjaminmoore.com/WebServices/prod/assets/production/datasheets/TDS_WPS-1000/WPS-1000_TDS_CE.pdf</x:v>
+      </x:c>
+      <x:c r="X55" t="str">
+        <x:v>Flat=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/insl-x-WPS-1000FR_SDS_EN.pdf?raw=true</x:v>
+      </x:c>
+      <x:c r="Z55" t="str">
+        <x:v>Flat=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/insl-x-WPS-1000_TDS_CE.pdf?raw=true</x:v>
       </x:c>
     </x:row>
     <x:row r="56">

</xml_diff>

<commit_message>
Add manufacturer SDS and TDS batch 037-039
</commit_message>
<xml_diff>
--- a/products_categories_descriptions_documents_working.xlsx
+++ b/products_categories_descriptions_documents_working.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" r:id="Re01872e8fd1547f3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" r:id="R4c452d58d3a94e99"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -3915,6 +3915,12 @@
       <x:c r="W56" t="str">
         <x:v>Semi Gloss=https://media.benjaminmoore.com/WebServices/prod/assets/production/datasheets/Pool_Paint_Faqs/CAE%20Pool%20Paint%20FAQs.pdf</x:v>
       </x:c>
+      <x:c r="X56" t="str">
+        <x:v>Semi Gloss=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/insl-x-WR-1023F_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/insl-x-WR-1024F_3001432_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/insl-x-WR-1019F_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/insl-x-WR-1020F_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/insl-x-WR-1010F_SDS_EN.pdf?raw=true</x:v>
+      </x:c>
+      <x:c r="Z56" t="str">
+        <x:v>Semi Gloss=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/insl-x-WR-10XX_TDS_CE.pdf?raw=true</x:v>
+      </x:c>
     </x:row>
     <x:row r="57">
       <x:c r="A57" t="str">
@@ -3976,6 +3982,12 @@
       <x:c r="W57" t="str">
         <x:v>Satin=https://media.benjaminmoore.com/WebServices/prod/assets/production/datasheets/TDS_RP-27XX/RP-27XX_TDS_CAE.pdf</x:v>
       </x:c>
+      <x:c r="X57" t="str">
+        <x:v>Satin=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/insl-x-RP-2719F_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/insl-x-RP-2720F_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/insl-x-RP-2723F_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/insl-x-RP-2724F_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/insl-x-RP-2710F_SDS_EN.pdf?raw=true</x:v>
+      </x:c>
+      <x:c r="Z57" t="str">
+        <x:v>Satin=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/insl-x-RP-27XX_TDS_CAE.pdf?raw=true</x:v>
+      </x:c>
     </x:row>
     <x:row r="58">
       <x:c r="A58" t="str">
@@ -4036,6 +4048,12 @@
       </x:c>
       <x:c r="W58" t="str">
         <x:v>Semi Gloss=https://media.benjaminmoore.com/WebServices/prod/assets/production/datasheets/TDS_IG-40XX/IG-40XX_TDS_CAE.pdf</x:v>
+      </x:c>
+      <x:c r="X58" t="str">
+        <x:v>Semi Gloss=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/insl-x-IG-4020F_EN_SDS.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/insl-x-IG-40BSF_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/insl-x-IG-4042F_EN_SDS.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/insl-x-IG-4001F_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/insl-x-IG-4024F_EN_SDS.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/insl-x-IG-4010F_SDS_EN.pdf?raw=true</x:v>
+      </x:c>
+      <x:c r="Z58" t="str">
+        <x:v>Semi Gloss=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/insl-x-IG-40XX_TDS_CAE.pdf?raw=true</x:v>
       </x:c>
     </x:row>
     <x:row r="59">

</xml_diff>

<commit_message>
Add manufacturer SDS and TDS batch 040-042
</commit_message>
<xml_diff>
--- a/products_categories_descriptions_documents_working.xlsx
+++ b/products_categories_descriptions_documents_working.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" r:id="R4c452d58d3a94e99"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" r:id="Rd37a9c02ee954c64"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2760,6 +2760,12 @@
       <x:c r="W37" t="str">
         <x:v>Gloss=https://media.benjaminmoore.com/WebServices/prod/assets/production/datasheets/TDS_V300/V300_TDS_CAE.pdf</x:v>
       </x:c>
+      <x:c r="X37" t="str">
+        <x:v>Gloss=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-HP3000-01FR_SDS_EN.pdf?raw=true</x:v>
+      </x:c>
+      <x:c r="Z37" t="str">
+        <x:v>Gloss=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/benjamin-moore-V300_TDS_CAE.pdf?raw=true</x:v>
+      </x:c>
     </x:row>
     <x:row r="38">
       <x:c r="A38" t="str">
@@ -2878,6 +2884,12 @@
       <x:c r="W39" t="str">
         <x:v>Semi Gloss=https://media.benjaminmoore.com/WebServices/prod/assets/production/datasheets/TDS_HP3410/HP3410_TDS_CE.pdf</x:v>
       </x:c>
+      <x:c r="X39" t="str">
+        <x:v>Semi Gloss=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-HP3410-9XFR_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-HP3410-8XFR_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-HP3410-7XFR_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-HP3410-01FR_SDS_EN.pdf?raw=true|Eggshell=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-HP3420-8XFR_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-HP3420-01FR_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-HP3420-7XFR_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-HP3420-9XFR_SDS_EN.pdf?raw=true</x:v>
+      </x:c>
+      <x:c r="Z39" t="str">
+        <x:v>Semi Gloss=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/benjamin-moore-HP3410_TDS_CE.pdf?raw=true</x:v>
+      </x:c>
     </x:row>
     <x:row r="40">
       <x:c r="A40" t="str">
@@ -3107,6 +3119,12 @@
       </x:c>
       <x:c r="W43" t="str">
         <x:v>Primer=https://media.benjaminmoore.com/WebServices/prod/assets/production/datasheets/TDS_HP1100/HP1100-20_TDS_CE.pdf?raw=true|Primer=https://media.benjaminmoore.com/WebServices/prod/assets/production/datasheets/TDS_HP1100/HP1100-01_TDS_CE.pdf?raw=true</x:v>
+      </x:c>
+      <x:c r="X43" t="str">
+        <x:v>Primer=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-HP1100-20FR_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-HP1100-01FR_SDS_EN.pdf?raw=true</x:v>
+      </x:c>
+      <x:c r="Z43" t="str">
+        <x:v>Primer=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/benjamin-moore-HP1100-20_TDS_CE.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/benjamin-moore-HP1100-01_TDS_CE.pdf?raw=true</x:v>
       </x:c>
     </x:row>
     <x:row r="44">

</xml_diff>

<commit_message>
Add manufacturer SDS and TDS batch 043-045
</commit_message>
<xml_diff>
--- a/products_categories_descriptions_documents_working.xlsx
+++ b/products_categories_descriptions_documents_working.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" r:id="Rd37a9c02ee954c64"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" r:id="R83a28589305340e3"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -3185,6 +3185,12 @@
       <x:c r="W44" t="str">
         <x:v>Sealer=https://media.benjaminmoore.com/WebServices/prod/assets/production/datasheets/TDS_HP1270/HP1270_TDS_CE.pdf?raw=true</x:v>
       </x:c>
+      <x:c r="X44" t="str">
+        <x:v>Sealer=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-HP1270-00FR_SDS_EN.pdf?raw=true</x:v>
+      </x:c>
+      <x:c r="Z44" t="str">
+        <x:v>Sealer=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/benjamin-moore-HP1270_TDS_CE.pdf?raw=true</x:v>
+      </x:c>
     </x:row>
     <x:row r="45">
       <x:c r="A45" t="str">
@@ -3244,6 +3250,12 @@
       <x:c r="W45" t="str">
         <x:v>Primer=https://media.benjaminmoore.com/WebServices/prod/assets/production/datasheets/TDS_HP1320/HP1320_TDS_CE.pdf?raw=true</x:v>
       </x:c>
+      <x:c r="X45" t="str">
+        <x:v>Primer=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-HP1320-70FR_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-HP1320-20FR_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-HP1320-01FR_SDS_EN.pdf?raw=true</x:v>
+      </x:c>
+      <x:c r="Z45" t="str">
+        <x:v>Primer=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/benjamin-moore-HP1320_TDS_CE.pdf?raw=true</x:v>
+      </x:c>
     </x:row>
     <x:row r="46">
       <x:c r="A46" t="str">
@@ -3302,6 +3314,12 @@
       </x:c>
       <x:c r="W46" t="str">
         <x:v>Primer=https://media.benjaminmoore.com/WebServices/prod/assets/production/datasheets/TDS_HP1420/HP1420_TDS_CE.pdf</x:v>
+      </x:c>
+      <x:c r="X46" t="str">
+        <x:v>Primer=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-HP1420-70FR_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-HP1420-20FR_SDS_EN.pdf?raw=true</x:v>
+      </x:c>
+      <x:c r="Z46" t="str">
+        <x:v>Primer=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/benjamin-moore-HP1420_TDS_CE.pdf?raw=true</x:v>
       </x:c>
     </x:row>
     <x:row r="47">

</xml_diff>

<commit_message>
Add manufacturer SDS and TDS batch 046-048
</commit_message>
<xml_diff>
--- a/products_categories_descriptions_documents_working.xlsx
+++ b/products_categories_descriptions_documents_working.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" r:id="R83a28589305340e3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" r:id="R021b5e14ab5f4694"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -3380,6 +3380,12 @@
       <x:c r="W47" t="str">
         <x:v>Primer=https://media.benjaminmoore.com/WebServices/prod/assets/production/datasheets/TDS_HP1550/HP1550_TDS_CE.pdf?raw=true</x:v>
       </x:c>
+      <x:c r="X47" t="str">
+        <x:v>Primer=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-HP1550-90FR_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-HP1550-00FR_SDS_EN.pdf?raw=true</x:v>
+      </x:c>
+      <x:c r="Z47" t="str">
+        <x:v>Primer=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/benjamin-moore-HP1550_TDS_CE.pdf?raw=true</x:v>
+      </x:c>
     </x:row>
     <x:row r="48">
       <x:c r="A48" t="str">
@@ -3439,6 +3445,12 @@
       <x:c r="W48" t="str">
         <x:v>Primer=https://media.benjaminmoore.com/WebServices/prod/assets/production/datasheets/TDS_HP1750/HP1750_TDS_CE.pdf?raw=true</x:v>
       </x:c>
+      <x:c r="X48" t="str">
+        <x:v>Primer=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-HP1750-00FR_SDS_EN.pdf?raw=true</x:v>
+      </x:c>
+      <x:c r="Z48" t="str">
+        <x:v>Primer=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/benjamin-moore-HP1750_TDS_CE.pdf?raw=true</x:v>
+      </x:c>
     </x:row>
     <x:row r="49">
       <x:c r="A49" t="str">
@@ -3499,6 +3511,12 @@
       </x:c>
       <x:c r="W49" t="str">
         <x:v>Gloss=https://media.benjaminmoore.com/WebServices/prod/assets/production/datasheets/TDS_HP4000/HP4000_TDS_CE.pdf?raw=true</x:v>
+      </x:c>
+      <x:c r="X49" t="str">
+        <x:v>Gloss=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-HP4000-75FR_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-HP4000-80FR_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-HP4000-90FR_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-HP4000-92FR_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-HP4000-91FR_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-HP4000-00FR_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-HP4000-9BFR_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-HP4000-8BFR_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-HP4000-20FR_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-HP4000-10FR_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-HP4000-70FR_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-HP4000-7BFR_SDS_EN.pdf?raw=true</x:v>
+      </x:c>
+      <x:c r="Z49" t="str">
+        <x:v>Gloss=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/benjamin-moore-HP4000_TDS_CE.pdf?raw=true</x:v>
       </x:c>
     </x:row>
     <x:row r="50">

</xml_diff>

<commit_message>
Add manufacturer SDS and TDS batch 049-050
</commit_message>
<xml_diff>
--- a/products_categories_descriptions_documents_working.xlsx
+++ b/products_categories_descriptions_documents_working.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" r:id="R021b5e14ab5f4694"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" r:id="Rc0ce7eadbcbf457a"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -3579,6 +3579,12 @@
       <x:c r="W50" t="str">
         <x:v>Satin=https://media.benjaminmoore.com/WebServices/prod/assets/production/datasheets/TDS_HP4100/HP4100_TDS_CE.pdf?raw=true</x:v>
       </x:c>
+      <x:c r="X50" t="str">
+        <x:v>Satin=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-HP4100-75FR_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-HP4100-80FR_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-HP4100-90FR_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-HP4100-9BFR_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-HP4100-00FR_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-HP4100-8BFR_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-HP4100-70FR_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-HP4100-7BFR_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-HP4100-01FR_SDS_EN.pdf?raw=true</x:v>
+      </x:c>
+      <x:c r="Z50" t="str">
+        <x:v>Satin=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/benjamin-moore-HP4100_TDS_CE.pdf?raw=true</x:v>
+      </x:c>
     </x:row>
     <x:row r="51">
       <x:c r="A51" t="str">
@@ -3639,6 +3645,12 @@
       </x:c>
       <x:c r="W51" t="str">
         <x:v>Gloss=https://media.benjaminmoore.com/WebServices/prod/assets/production/datasheets/TDS_HP4300/HP4300_TDS_CE.pdf?raw=true</x:v>
+      </x:c>
+      <x:c r="X51" t="str">
+        <x:v>Gloss=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-HP4300-90FR_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-HP4300-00FR_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-HP4300-52FR_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-HP4300-70FR_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-HP4300-01FR_SDS_EN.pdf?raw=true</x:v>
+      </x:c>
+      <x:c r="Z51" t="str">
+        <x:v>Gloss=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/benjamin-moore-HP4300_TDS_CE.pdf?raw=true</x:v>
       </x:c>
     </x:row>
     <x:row r="52">

</xml_diff>

<commit_message>
Add researched manufacturer SDS and TDS batch 051-053
</commit_message>
<xml_diff>
--- a/products_categories_descriptions_documents_working.xlsx
+++ b/products_categories_descriptions_documents_working.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" r:id="Rc0ce7eadbcbf457a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" r:id="R737cf79d900143ad"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2823,6 +2823,12 @@
       <x:c r="U38" t="str"/>
       <x:c r="V38" t="str"/>
       <x:c r="W38" t="str"/>
+      <x:c r="X38" t="str">
+        <x:v>Gloss=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-HP3300-10FR_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-HP3300-01FR_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-HP3300-20FR_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-HP3300-7XFR_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-HP3300-80FR_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-HP3300-9XFR_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-HP3300-8XFR_SDS_EN.pdf?raw=true|Satin=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-HP3320-01FR_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-HP3320-62FR_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-HP3320-7XFR_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-HP3320-80FR_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-HP3320-8XFR_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-HP3320-9XFR_SDS_EN.pdf?raw=true</x:v>
+      </x:c>
+      <x:c r="Z38" t="str">
+        <x:v>Gloss=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/benjamin-moore-HP3300_TDS_CE.pdf?raw=true|Satin=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/benjamin-moore-HP3320_TDS_CE.pdf?raw=true</x:v>
+      </x:c>
     </x:row>
     <x:row r="39">
       <x:c r="A39" t="str">
@@ -2947,6 +2953,12 @@
       <x:c r="U40" t="str"/>
       <x:c r="V40" t="str"/>
       <x:c r="W40" t="str"/>
+      <x:c r="X40" t="str">
+        <x:v>Gloss=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-HP3900-01FR_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-HP3900-10FR_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-HP3900-20FR_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-HP3900-7XFR_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-HP3900-80FR_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-HP3900-8XFR_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-HP3900-9XFR_SDS_EN.pdf?raw=true|Satin=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-HP3920-62FR_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-HP3920-01FR_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-HP3920-7XFR_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-HP3920-80FR_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-HP3920-9XFR_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-HP3920-8XFR_SDS_EN.pdf?raw=true</x:v>
+      </x:c>
+      <x:c r="Z40" t="str">
+        <x:v>Gloss=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/benjamin-moore-HP3900_TDS_CE.pdf?raw=true|Satin=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/benjamin-moore-HP3920_TDS_CE.pdf?raw=true</x:v>
+      </x:c>
     </x:row>
     <x:row r="41">
       <x:c r="A41" t="str">
@@ -3004,6 +3016,12 @@
       <x:c r="U41" t="str"/>
       <x:c r="V41" t="str"/>
       <x:c r="W41" t="str"/>
+      <x:c r="X41" t="str">
+        <x:v>Gloss=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-HP5000-00FR_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-HP5000-01FR_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-HP5000-7BFR_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-HP5000-80FR_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-HP5000-8BFR_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-HP5000-90FR_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-HP5000-9BFR_SDS_EN.pdf?raw=true|Semi Gloss=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-HP5010-7BFR_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-HP5010-90FR_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-HP5010-8BFR_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-HP5010-9BFR_SDS_EN.pdf?raw=true</x:v>
+      </x:c>
+      <x:c r="Z41" t="str">
+        <x:v>Gloss=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/benjamin-moore-HP5000_TDS_CE.pdf?raw=true|Semi Gloss=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/benjamin-moore-HP5010_TDS_CE.pdf?raw=true</x:v>
+      </x:c>
     </x:row>
     <x:row r="42">
       <x:c r="A42" t="str">

</xml_diff>

<commit_message>
Add manufacturer SDS and TDS batch 054-056
</commit_message>
<xml_diff>
--- a/products_categories_descriptions_documents_working.xlsx
+++ b/products_categories_descriptions_documents_working.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" r:id="R737cf79d900143ad"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" r:id="Rc221016421ee4e41"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -471,6 +471,9 @@
       <x:c r="U2" t="str"/>
       <x:c r="V2" t="str"/>
       <x:c r="W2" t="str"/>
+      <x:c r="X2" t="str">
+        <x:v>Colour Sample=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-K2001X_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-K2003X_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-K2002X_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-K2004X_SDS_EN.pdf?raw=true</x:v>
+      </x:c>
     </x:row>
     <x:row r="3">
       <x:c r="A3" t="str">
@@ -526,6 +529,12 @@
       <x:c r="U3" t="str"/>
       <x:c r="V3" t="str"/>
       <x:c r="W3" t="str"/>
+      <x:c r="X3" t="str">
+        <x:v>Translucent=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-K69140_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-K69165_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-K69160_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-K69110_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-K69120_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-K69130_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-K69178_SDS_EN.pdf?raw=true|Semi-Transparent=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-K69206_SDS_EN.pdf?raw=true|Semi-Solid=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-K69301_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-K69306_SDS_EN.pdf?raw=true|Solid=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-K6941X_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-K6942X_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-K6943X_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-K6944X_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-K69401_SDS_EN.pdf?raw=true</x:v>
+      </x:c>
+      <x:c r="Z3" t="str">
+        <x:v>Translucent=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/benjamin-moore-K691_TDS_CE.pdf?raw=true|Semi-Transparent=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/benjamin-moore-K692_TDS_CE.pdf?raw=true|Semi-Solid=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/benjamin-moore-K693_TDS_CE.pdf?raw=true|Solid=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/benjamin-moore-K694_TDS_CE.pdf?raw=true</x:v>
+      </x:c>
     </x:row>
     <x:row r="4">
       <x:c r="A4" t="str">
@@ -3079,6 +3088,12 @@
       <x:c r="U42" t="str"/>
       <x:c r="V42" t="str"/>
       <x:c r="W42" t="str"/>
+      <x:c r="X42" t="str">
+        <x:v>Gloss=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-HP5700-7BFR_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-HP5700-8BFR_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-HP5700-90FR_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-HP5700-9BFR_SDS_EN.pdf?raw=true|Satin=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-HP5720-7BFR_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-HP5720-9BFR_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-HP5720-8BFR_SDS_EN.pdf?raw=true, https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-HP5720-80FR_SDS_EN.pdf?raw=true</x:v>
+      </x:c>
+      <x:c r="Z42" t="str">
+        <x:v>Gloss=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/benjamin-moore-HP5700_TDS_CE.pdf?raw=true|Satin=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/benjamin-moore-HP5720_TDS_CE.pdf?raw=true</x:v>
+      </x:c>
     </x:row>
     <x:row r="43">
       <x:c r="A43" t="str">

</xml_diff>

<commit_message>
Add manufacturer SDS and TDS batch 057-059
</commit_message>
<xml_diff>
--- a/products_categories_descriptions_documents_working.xlsx
+++ b/products_categories_descriptions_documents_working.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" r:id="Rc221016421ee4e41"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" r:id="Rfd1e145d2fcc48f6"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -6798,6 +6798,12 @@
       <x:c r="U112" t="str"/>
       <x:c r="V112" t="str"/>
       <x:c r="W112" t="str"/>
+      <x:c r="X112" t="str">
+        <x:v>250 VOC=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/messmer-s-SDS-CDSO-2015.pdf?raw=true|550 VOC=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/messmer-s-SDS-DSO-2015.pdf?raw=true</x:v>
+      </x:c>
+      <x:c r="Z112" t="str">
+        <x:v>Deck and Siding Stain=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/messmer-s-td-dso.pdf?raw=true</x:v>
+      </x:c>
     </x:row>
     <x:row r="113">
       <x:c r="A113" t="str">
@@ -8464,6 +8470,12 @@
       <x:c r="U146" t="str"/>
       <x:c r="V146" t="str"/>
       <x:c r="W146" t="str"/>
+      <x:c r="X146" t="str">
+        <x:v>Gallon=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/old-masters-11201_AGHS_EN.pdf?raw=true|Quart=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/old-masters-11204_AGHS_EN.pdf?raw=true|Half Pint=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/old-masters-11216_AGHS_EN.pdf?raw=true</x:v>
+      </x:c>
+      <x:c r="Z146" t="str">
+        <x:v>Wiping Stain=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/old-masters-OM-Wiping-Stain-Data-Sheet.pdf?raw=true</x:v>
+      </x:c>
     </x:row>
     <x:row r="147">
       <x:c r="A147" t="str">
@@ -8562,6 +8574,12 @@
       <x:c r="U148" t="str"/>
       <x:c r="V148" t="str"/>
       <x:c r="W148" t="str"/>
+      <x:c r="X148" t="str">
+        <x:v>Gallon=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/old-masters-51101_AGHS_EN.pdf?raw=true|Quart=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/old-masters-51104_AGHS_EN.pdf?raw=true</x:v>
+      </x:c>
+      <x:c r="Z148" t="str">
+        <x:v>Wood Conditioner=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/old-masters-OM-Wood-Conditioner-Data-Sheet.pdf?raw=true</x:v>
+      </x:c>
     </x:row>
     <x:row r="149">
       <x:c r="A149" t="str">

</xml_diff>

<commit_message>
Add manufacturer SDS and TDS batch 060-062
</commit_message>
<xml_diff>
--- a/products_categories_descriptions_documents_working.xlsx
+++ b/products_categories_descriptions_documents_working.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" r:id="Rfd1e145d2fcc48f6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" r:id="R7ea233b87e724437"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -8629,6 +8629,12 @@
       <x:c r="U149" t="str"/>
       <x:c r="V149" t="str"/>
       <x:c r="W149" t="str"/>
+      <x:c r="X149" t="str">
+        <x:v>Flat Gallon=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/old-masters-72001_AGHS_EN.pdf?raw=true|Satin Gallon=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/old-masters-72101_AGHS_EN.pdf?raw=true|Semi-Gloss Gallon=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/old-masters-72201_AGHS_EN.pdf?raw=true|Gloss Gallon=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/old-masters-72301_AGHS_EN.pdf?raw=true</x:v>
+      </x:c>
+      <x:c r="Z149" t="str">
+        <x:v>Masters Armor=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/old-masters-OM-Masters-Armor-Data-Sheet.pdf?raw=true</x:v>
+      </x:c>
     </x:row>
     <x:row r="150">
       <x:c r="A150" t="str">
@@ -8678,6 +8684,12 @@
       <x:c r="U150" t="str"/>
       <x:c r="V150" t="str"/>
       <x:c r="W150" t="str"/>
+      <x:c r="X150" t="str">
+        <x:v>Natural Gallon=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/old-masters-76101_AGHS_EN.pdf?raw=true|Natural Quart=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/old-masters-76104_AGHS_EN.pdf?raw=true</x:v>
+      </x:c>
+      <x:c r="Z150" t="str">
+        <x:v>Water-Based Wood Stain=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/old-masters-OM-Water-Based-Stain-Data-Sheet.pdf?raw=true</x:v>
+      </x:c>
     </x:row>
     <x:row r="151">
       <x:c r="A151" t="str">
@@ -8727,6 +8739,12 @@
       <x:c r="U151" t="str"/>
       <x:c r="V151" t="str"/>
       <x:c r="W151" t="str"/>
+      <x:c r="X151" t="str">
+        <x:v>Natural Quart=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/old-masters-80104_AGHS_EN.pdf?raw=true</x:v>
+      </x:c>
+      <x:c r="Z151" t="str">
+        <x:v>Gel Stain=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/old-masters-OM-Gel-Stain-Data-Sheet.pdf?raw=true</x:v>
+      </x:c>
     </x:row>
     <x:row r="152">
       <x:c r="A152" t="str">

</xml_diff>

<commit_message>
Add manufacturer SDS and TDS batch 063-065
</commit_message>
<xml_diff>
--- a/products_categories_descriptions_documents_working.xlsx
+++ b/products_categories_descriptions_documents_working.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" r:id="R7ea233b87e724437"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" r:id="R5fa4abe23abb42dc"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -9284,6 +9284,12 @@
       <x:c r="U162" t="str"/>
       <x:c r="V162" t="str"/>
       <x:c r="W162" t="str"/>
+      <x:c r="X162" t="str">
+        <x:v>369 g Aerosol=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/zinsser-254168.pdf?raw=true</x:v>
+      </x:c>
+      <x:c r="Z162" t="str">
+        <x:v>13 oz Aerosol=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/zinsser-OLS-02_Odorless_Primer_Sealer_Stain_Blocker_TDS.ashx.pdf?raw=true</x:v>
+      </x:c>
     </x:row>
     <x:row r="163">
       <x:c r="A163" t="str">
@@ -9333,6 +9339,12 @@
       <x:c r="U163" t="str"/>
       <x:c r="V163" t="str"/>
       <x:c r="W163" t="str"/>
+      <x:c r="X163" t="str">
+        <x:v>946 mL=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/zinsser-256185.pdf?raw=true|3.7 L=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/zinsser-256184.pdf?raw=true|18.9 L=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/zinsser-256188.pdf?raw=true</x:v>
+      </x:c>
+      <x:c r="Z163" t="str">
+        <x:v>Cover Stain=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/zinsser-CVS-13-Zinsser-Cover-Stain-TDS-EN-24.pdf?raw=true</x:v>
+      </x:c>
     </x:row>
     <x:row r="164">
       <x:c r="A164" t="str">
@@ -9382,6 +9394,12 @@
       <x:c r="U164" t="str"/>
       <x:c r="V164" t="str"/>
       <x:c r="W164" t="str"/>
+      <x:c r="X164" t="str">
+        <x:v>369 g Aerosol=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/zinsser-Z03618.pdf?raw=true</x:v>
+      </x:c>
+      <x:c r="Z164" t="str">
+        <x:v>Cover Stain Aerosol=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/zinsser-CVS-09_Cover_Stain_Oil-Base_Primer_Spray_TDS_1.ashx.pdf?raw=true</x:v>
+      </x:c>
     </x:row>
     <x:row r="165">
       <x:c r="A165" t="str">

</xml_diff>

<commit_message>
Add manufacturer SDS and TDS batch 066-068
</commit_message>
<xml_diff>
--- a/products_categories_descriptions_documents_working.xlsx
+++ b/products_categories_descriptions_documents_working.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" r:id="R5fa4abe23abb42dc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" r:id="R4e08bd980bfc45e0"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -9449,6 +9449,12 @@
       <x:c r="U165" t="str"/>
       <x:c r="V165" t="str"/>
       <x:c r="W165" t="str"/>
+      <x:c r="X165" t="str">
+        <x:v>473 mL=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/zinsser-Z00918.pdf?raw=true|946 mL=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/zinsser-Z00914.pdf?raw=true|3.7 L=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/zinsser-Z00911.pdf?raw=true|18.9 L=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/zinsser-Z00910.pdf?raw=true</x:v>
+      </x:c>
+      <x:c r="Z165" t="str">
+        <x:v>B-I-N Liquid=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/zinsser-BIN-03-Zinsser-B-I-N-Shellac-Base-Primer-TDS-EN-24.pdf?raw=true</x:v>
+      </x:c>
     </x:row>
     <x:row r="166">
       <x:c r="A166" t="str">
@@ -9498,6 +9504,12 @@
       <x:c r="U166" t="str"/>
       <x:c r="V166" t="str"/>
       <x:c r="W166" t="str"/>
+      <x:c r="X166" t="str">
+        <x:v>369 g Aerosol=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/zinsser-Z01018.pdf?raw=true</x:v>
+      </x:c>
+      <x:c r="Z166" t="str">
+        <x:v>B-I-N Aerosol=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/zinsser-BIN-03-Zinsser-B-I-N-Shellac-Base-Primer-TDS-EN-24.pdf?raw=true</x:v>
+      </x:c>
     </x:row>
     <x:row r="167">
       <x:c r="A167" t="str">
@@ -9547,6 +9559,12 @@
       <x:c r="U167" t="str"/>
       <x:c r="V167" t="str"/>
       <x:c r="W167" t="str"/>
+      <x:c r="X167" t="str">
+        <x:v>946 mL White=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/zinsser-Z02014.pdf?raw=true|3.78 L White=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/zinsser-Z02012.pdf?raw=true|18.9 L White=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/zinsser-Z02010.pdf?raw=true</x:v>
+      </x:c>
+      <x:c r="Z167" t="str">
+        <x:v>Bulls Eye 1-2-3 White Liquid=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/zinsser-BEY123-01-Zinsser-Bulls-Eye-1-2-3-Water-based-Primer-TDS-EN-21.pdf?raw=true</x:v>
+      </x:c>
     </x:row>
     <x:row r="168">
       <x:c r="A168" t="str">

</xml_diff>

<commit_message>
Add manufacturer SDS and TDS batch 069-071
</commit_message>
<xml_diff>
--- a/products_categories_descriptions_documents_working.xlsx
+++ b/products_categories_descriptions_documents_working.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" r:id="R4e08bd980bfc45e0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" r:id="Ra5d7017ed84544d7"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -9614,6 +9614,12 @@
       <x:c r="U168" t="str"/>
       <x:c r="V168" t="str"/>
       <x:c r="W168" t="str"/>
+      <x:c r="X168" t="str">
+        <x:v>340 g Aerosol Gloss Grey=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/tremclad-27028B522.pdf?raw=true</x:v>
+      </x:c>
+      <x:c r="Z168" t="str">
+        <x:v>Tremclad Rust Paint Aerosol=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/tremclad-TRM-02-Tremclad-Rust-Paint-Aerosol-TDS-Canada.pdf?raw=true</x:v>
+      </x:c>
     </x:row>
     <x:row r="169">
       <x:c r="A169" t="str">
@@ -9663,6 +9669,9 @@
       <x:c r="U169" t="str"/>
       <x:c r="V169" t="str"/>
       <x:c r="W169" t="str"/>
+      <x:c r="X169" t="str">
+        <x:v>237 mL Flat Black=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/tremclad-29300125.pdf?raw=true|946 mL Flat Black=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/tremclad-254898.pdf?raw=true|340 g Aerosol Flat Black=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/tremclad-29300522.pdf?raw=true</x:v>
+      </x:c>
     </x:row>
     <x:row r="170">
       <x:c r="A170" t="str">
@@ -9712,6 +9721,9 @@
       <x:c r="U170" t="str"/>
       <x:c r="V170" t="str"/>
       <x:c r="W170" t="str"/>
+      <x:c r="X170" t="str">
+        <x:v>237 mL Gloss Yellow=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/tremclad-27097X125.pdf?raw=true|946 mL Gloss Yellow=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/tremclad-254922.pdf?raw=true|3.78 L Gloss Yellow=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/tremclad-27097X155.pdf?raw=true</x:v>
+      </x:c>
     </x:row>
     <x:row r="171">
       <x:c r="A171" t="str">

</xml_diff>

<commit_message>
Add manufacturer SDS batch 072-074
</commit_message>
<xml_diff>
--- a/products_categories_descriptions_documents_working.xlsx
+++ b/products_categories_descriptions_documents_working.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" r:id="Ra5d7017ed84544d7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" r:id="R6ad70f817faf45ca"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -9773,6 +9773,9 @@
       <x:c r="U171" t="str"/>
       <x:c r="V171" t="str"/>
       <x:c r="W171" t="str"/>
+      <x:c r="X171" t="str">
+        <x:v>237 mL Semi-Gloss White=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/tremclad-270S25X125.pdf?raw=true|946 mL Semi-Gloss White=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/tremclad-254933.pdf?raw=true|3.78 L Semi-Gloss White=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/tremclad-270S25X155.pdf?raw=true</x:v>
+      </x:c>
     </x:row>
     <x:row r="172">
       <x:c r="A172" t="str">
@@ -9822,6 +9825,9 @@
       <x:c r="U172" t="str"/>
       <x:c r="V172" t="str"/>
       <x:c r="W172" t="str"/>
+      <x:c r="X172" t="str">
+        <x:v>237 mL Flat White=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/tremclad-27061X125.pdf?raw=true|946 mL Flat White=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/tremclad-254929.pdf?raw=true|3.78 L Flat White=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/tremclad-27061X155.pdf?raw=true</x:v>
+      </x:c>
     </x:row>
     <x:row r="173">
       <x:c r="A173" t="str">
@@ -9871,6 +9877,9 @@
       <x:c r="U173" t="str"/>
       <x:c r="V173" t="str"/>
       <x:c r="W173" t="str"/>
+      <x:c r="X173" t="str">
+        <x:v>237 mL Gloss Recreational White=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/tremclad-27032X125.pdf?raw=true|946 mL Gloss Recreational White=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/tremclad-254910.pdf?raw=true|3.78 L Gloss Recreational White=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/tremclad-27032X155.pdf?raw=true</x:v>
+      </x:c>
     </x:row>
     <x:row r="174">
       <x:c r="A174" t="str">

</xml_diff>

<commit_message>
Add manufacturer SDS batch 075-077
</commit_message>
<xml_diff>
--- a/products_categories_descriptions_documents_working.xlsx
+++ b/products_categories_descriptions_documents_working.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" r:id="R6ad70f817faf45ca"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" r:id="R38c8fa26d70c4c43"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -9929,6 +9929,9 @@
       <x:c r="U174" t="str"/>
       <x:c r="V174" t="str"/>
       <x:c r="W174" t="str"/>
+      <x:c r="X174" t="str">
+        <x:v>946 mL Gloss Real Orange=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/tremclad-369814.pdf?raw=true|3.78 L Gloss Real Orange=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/tremclad-27007X155.pdf?raw=true</x:v>
+      </x:c>
     </x:row>
     <x:row r="175">
       <x:c r="A175" t="str">
@@ -9978,6 +9981,9 @@
       <x:c r="U175" t="str"/>
       <x:c r="V175" t="str"/>
       <x:c r="W175" t="str"/>
+      <x:c r="X175" t="str">
+        <x:v>946 mL Gloss Medium Blue=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/tremclad-254905.pdf?raw=true|3.78 L Gloss Medium Blue=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/tremclad-27009X155.pdf?raw=true</x:v>
+      </x:c>
     </x:row>
     <x:row r="176">
       <x:c r="A176" t="str">
@@ -10027,6 +10033,9 @@
       <x:c r="U176" t="str"/>
       <x:c r="V176" t="str"/>
       <x:c r="W176" t="str"/>
+      <x:c r="X176" t="str">
+        <x:v>946 mL Gloss John Deere Green=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/tremclad-254913.pdf?raw=true|3.78 L Gloss John Deere Green=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/tremclad-27039X155.pdf?raw=true</x:v>
+      </x:c>
     </x:row>
     <x:row r="177">
       <x:c r="A177" t="str">

</xml_diff>

<commit_message>
Add manufacturer SDS batch 078-080
</commit_message>
<xml_diff>
--- a/products_categories_descriptions_documents_working.xlsx
+++ b/products_categories_descriptions_documents_working.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" r:id="R38c8fa26d70c4c43"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" r:id="R2e665110f0c948d4"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -10085,6 +10085,9 @@
       <x:c r="U177" t="str"/>
       <x:c r="V177" t="str"/>
       <x:c r="W177" t="str"/>
+      <x:c r="X177" t="str">
+        <x:v>237 mL Gloss Grey=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/tremclad-27028X125.pdf?raw=true|946 mL Gloss Grey=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/tremclad-254908.pdf?raw=true|3.78 L Gloss Grey=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/tremclad-27028X155.pdf?raw=true</x:v>
+      </x:c>
     </x:row>
     <x:row r="178">
       <x:c r="A178" t="str">
@@ -10134,6 +10137,9 @@
       <x:c r="U178" t="str"/>
       <x:c r="V178" t="str"/>
       <x:c r="W178" t="str"/>
+      <x:c r="X178" t="str">
+        <x:v>237 mL Gloss Fire Red=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/tremclad-27049X125.pdf?raw=true|946 mL Gloss Fire Red=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/tremclad-254915.pdf?raw=true|3.78 L Gloss Fire Red=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/tremclad-27049X155.pdf?raw=true</x:v>
+      </x:c>
     </x:row>
     <x:row r="179">
       <x:c r="A179" t="str">
@@ -10183,6 +10189,9 @@
       <x:c r="U179" t="str"/>
       <x:c r="V179" t="str"/>
       <x:c r="W179" t="str"/>
+      <x:c r="X179" t="str">
+        <x:v>237 mL Gloss Dark Blue=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/tremclad-27067X125.pdf?raw=true|946 mL Gloss Dark Blue=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/tremclad-254916.pdf?raw=true|3.78 L Gloss Dark Blue=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/tremclad-27067X155.pdf?raw=true</x:v>
+      </x:c>
     </x:row>
     <x:row r="180">
       <x:c r="A180" t="str">

</xml_diff>

<commit_message>
Add manufacturer SDS batch 081-083
</commit_message>
<xml_diff>
--- a/products_categories_descriptions_documents_working.xlsx
+++ b/products_categories_descriptions_documents_working.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" r:id="R2e665110f0c948d4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" r:id="R676d819ba9c94ed1"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -10241,6 +10241,9 @@
       <x:c r="U180" t="str"/>
       <x:c r="V180" t="str"/>
       <x:c r="W180" t="str"/>
+      <x:c r="X180" t="str">
+        <x:v>237 mL Gloss Brown=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/tremclad-27095X125.pdf?raw=true|946 mL Gloss Brown=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/tremclad-254920.pdf?raw=true|3.78 L Gloss Brown=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/tremclad-27095X155.pdf?raw=true</x:v>
+      </x:c>
     </x:row>
     <x:row r="181">
       <x:c r="A181" t="str">
@@ -10290,6 +10293,9 @@
       <x:c r="U181" t="str"/>
       <x:c r="V181" t="str"/>
       <x:c r="W181" t="str"/>
+      <x:c r="X181" t="str">
+        <x:v>237 mL Semi-Gloss Black=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/tremclad-270S26X125.pdf?raw=true|946 mL Semi-Gloss Black=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/tremclad-254940.pdf?raw=true|3.78 L Semi-Gloss Black=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/tremclad-270S26X155.pdf?raw=true</x:v>
+      </x:c>
     </x:row>
     <x:row r="182">
       <x:c r="A182" t="str">
@@ -10339,6 +10345,9 @@
       <x:c r="U182" t="str"/>
       <x:c r="V182" t="str"/>
       <x:c r="W182" t="str"/>
+      <x:c r="X182" t="str">
+        <x:v>237 mL Gloss Black=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/tremclad-27026X125.pdf?raw=true|946 mL Gloss Black=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/tremclad-254926.pdf?raw=true|3.78 L Gloss Black=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/tremclad-27026X155.pdf?raw=true</x:v>
+      </x:c>
     </x:row>
     <x:row r="183">
       <x:c r="A183" t="str">

</xml_diff>

<commit_message>
Add manufacturer SDS batch 084-086
</commit_message>
<xml_diff>
--- a/products_categories_descriptions_documents_working.xlsx
+++ b/products_categories_descriptions_documents_working.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" r:id="R676d819ba9c94ed1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" r:id="Rb5327ac265f44e6c"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -10397,6 +10397,9 @@
       <x:c r="U183" t="str"/>
       <x:c r="V183" t="str"/>
       <x:c r="W183" t="str"/>
+      <x:c r="X183" t="str">
+        <x:v>237 mL Flat Black=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/tremclad-27048X125.pdf?raw=true|946 mL Flat Black=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/tremclad-254932.pdf?raw=true|3.78 L Flat Black=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/tremclad-27048X155.pdf?raw=true</x:v>
+      </x:c>
     </x:row>
     <x:row r="184">
       <x:c r="A184" t="str">
@@ -10446,6 +10449,9 @@
       <x:c r="U184" t="str"/>
       <x:c r="V184" t="str"/>
       <x:c r="W184" t="str"/>
+      <x:c r="X184" t="str">
+        <x:v>237 mL Gloss Aluminum=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/tremclad-27006X125.pdf?raw=true|946 mL Gloss Aluminum=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/tremclad-254904.pdf?raw=true|3.78 L Gloss Aluminum=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/tremclad-27006X155.pdf?raw=true</x:v>
+      </x:c>
     </x:row>
     <x:row r="185">
       <x:c r="A185" t="str">
@@ -10495,6 +10501,9 @@
       <x:c r="U185" t="str"/>
       <x:c r="V185" t="str"/>
       <x:c r="W185" t="str"/>
+      <x:c r="X185" t="str">
+        <x:v>3.78 L Flat Grey=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/tremclad-274103155.pdf?raw=true</x:v>
+      </x:c>
     </x:row>
     <x:row r="186">
       <x:c r="A186" t="str">

</xml_diff>

<commit_message>
Add manufacturer SDS and TDS batch 087-089
</commit_message>
<xml_diff>
--- a/products_categories_descriptions_documents_working.xlsx
+++ b/products_categories_descriptions_documents_working.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" r:id="Rb5327ac265f44e6c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" r:id="R21a80e00edb8485b"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -10553,6 +10553,9 @@
       <x:c r="U186" t="str"/>
       <x:c r="V186" t="str"/>
       <x:c r="W186" t="str"/>
+      <x:c r="X186" t="str">
+        <x:v>3.78 L Flat Red Oxide=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/tremclad-274102155.pdf?raw=true</x:v>
+      </x:c>
     </x:row>
     <x:row r="187">
       <x:c r="A187" t="str">
@@ -10602,6 +10605,12 @@
       <x:c r="U187" t="str"/>
       <x:c r="V187" t="str"/>
       <x:c r="W187" t="str"/>
+      <x:c r="X187" t="str">
+        <x:v>3.78 L White=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/zinsser-336961.pdf?raw=true|946 mL White=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/zinsser-336964.pdf?raw=true</x:v>
+      </x:c>
+      <x:c r="Z187" t="str">
+        <x:v>Mould Stop Primer=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/zinsser-336964_Mould-Stop-Primer-TDS-EN.ashx.pdf?raw=true</x:v>
+      </x:c>
     </x:row>
     <x:row r="188">
       <x:c r="A188" t="str">
@@ -10651,6 +10660,12 @@
       <x:c r="U188" t="str"/>
       <x:c r="V188" t="str"/>
       <x:c r="W188" t="str"/>
+      <x:c r="X188" t="str">
+        <x:v>369 g Aerosol White=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/zinsser-267189.pdf?raw=true</x:v>
+      </x:c>
+      <x:c r="Z188" t="str">
+        <x:v>Bulls Eye 1-2-3 Aerosol=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/zinsser-BEY123-01-Zinsser-Bulls-Eye-1-2-3-Water-based-Primer-TDS-EN-21.pdf?raw=true</x:v>
+      </x:c>
     </x:row>
     <x:row r="189">
       <x:c r="A189" t="str">

</xml_diff>

<commit_message>
Add manufacturer SDS and TDS batch 090-092
</commit_message>
<xml_diff>
--- a/products_categories_descriptions_documents_working.xlsx
+++ b/products_categories_descriptions_documents_working.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" r:id="R21a80e00edb8485b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" r:id="R16b9a103843f42bd"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -10715,6 +10715,9 @@
       <x:c r="U189" t="str"/>
       <x:c r="V189" t="str"/>
       <x:c r="W189" t="str"/>
+      <x:c r="X189" t="str">
+        <x:v>946 mL Flat Grey=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/tremclad-254895.pdf?raw=true</x:v>
+      </x:c>
     </x:row>
     <x:row r="190">
       <x:c r="A190" t="str">
@@ -10764,6 +10767,9 @@
       <x:c r="U190" t="str"/>
       <x:c r="V190" t="str"/>
       <x:c r="W190" t="str"/>
+      <x:c r="X190" t="str">
+        <x:v>946 mL Flat Red Oxide=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/tremclad-254894.pdf?raw=true</x:v>
+      </x:c>
     </x:row>
     <x:row r="191">
       <x:c r="A191" t="str">
@@ -10813,6 +10819,12 @@
       <x:c r="U191" t="str"/>
       <x:c r="V191" t="str"/>
       <x:c r="W191" t="str"/>
+      <x:c r="X191" t="str">
+        <x:v>946 mL White=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/zinsser-248264.pdf?raw=true|3.7 L White=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/zinsser-248263.pdf?raw=true</x:v>
+      </x:c>
+      <x:c r="Z191" t="str">
+        <x:v>Odorless Oil-Base Stain Blocker Liquid=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/zinsser-OLS-01_Odorless_Interior_Oil_Base_Stain_Blocker_TDS_2.ashx.pdf?raw=true</x:v>
+      </x:c>
     </x:row>
     <x:row r="192">
       <x:c r="A192" t="str">

</xml_diff>

<commit_message>
Add manufacturer SDS and TDS batch 093-095
</commit_message>
<xml_diff>
--- a/products_categories_descriptions_documents_working.xlsx
+++ b/products_categories_descriptions_documents_working.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" r:id="R16b9a103843f42bd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" r:id="R5e1b9c812d1243c0"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -10874,6 +10874,12 @@
       <x:c r="U192" t="str"/>
       <x:c r="V192" t="str"/>
       <x:c r="W192" t="str"/>
+      <x:c r="X192" t="str">
+        <x:v>946 mL Grey=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/zinsser-201746.pdf?raw=true|3.7 L Grey=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/zinsser-201791.pdf?raw=true</x:v>
+      </x:c>
+      <x:c r="Z192" t="str">
+        <x:v>Bulls Eye 1-2-3 Grey Primer=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/zinsser-BEY123-10_Bulls-Eye_1-2-3_Primer_For_All_Surfaces_TDS.ashx.pdf?raw=true</x:v>
+      </x:c>
     </x:row>
     <x:row r="193">
       <x:c r="A193" t="str">
@@ -10923,6 +10929,9 @@
       <x:c r="U193" t="str"/>
       <x:c r="V193" t="str"/>
       <x:c r="W193" t="str"/>
+      <x:c r="X193" t="str">
+        <x:v>237 mL Flat Leather Brown=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/tremclad-27091X125.pdf?raw=true|946 mL Flat Leather Brown=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/tremclad-254919.pdf?raw=true|3.78 L Flat Leather Brown=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/tremclad-27091X155.pdf?raw=true</x:v>
+      </x:c>
     </x:row>
     <x:row r="194">
       <x:c r="A194" t="str">
@@ -10972,6 +10981,9 @@
       <x:c r="U194" t="str"/>
       <x:c r="V194" t="str"/>
       <x:c r="W194" t="str"/>
+      <x:c r="X194" t="str">
+        <x:v>237 mL Gloss Green=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/tremclad-27029X125.pdf?raw=true|946 mL Gloss Green=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/tremclad-254909.pdf?raw=true|3.78 L Gloss Green=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/tremclad-27029X155.pdf?raw=true</x:v>
+      </x:c>
     </x:row>
     <x:row r="195">
       <x:c r="A195" t="str">

</xml_diff>

<commit_message>
Add manufacturer SDS and TDS batch 096-098
</commit_message>
<xml_diff>
--- a/products_categories_descriptions_documents_working.xlsx
+++ b/products_categories_descriptions_documents_working.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" r:id="R5e1b9c812d1243c0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" r:id="R1df7d6abc79948a7"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -11033,6 +11033,9 @@
       <x:c r="U195" t="str"/>
       <x:c r="V195" t="str"/>
       <x:c r="W195" t="str"/>
+      <x:c r="X195" t="str">
+        <x:v>237 mL Gloss White=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/tremclad-27025X125.pdf?raw=true|946 mL Gloss White=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/tremclad-254924.pdf?raw=true|3.78 L Gloss White=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/tremclad-27025X155.pdf?raw=true</x:v>
+      </x:c>
     </x:row>
     <x:row r="196">
       <x:c r="A196" t="str">
@@ -11870,6 +11873,12 @@
       <x:c r="U212" t="str"/>
       <x:c r="V212" t="str"/>
       <x:c r="W212" t="str"/>
+      <x:c r="X212" t="str">
+        <x:v>Flat / Satin / Semi-Gloss / Gloss=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/saman-SDS_SAM-505-SAM-535-SAM-565-SAM-595.pdf?raw=true</x:v>
+      </x:c>
+      <x:c r="Z212" t="str">
+        <x:v>Flat / Satin / Semi-Gloss / Gloss=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/saman-TDS-ANG_-SAM-505-535-565-595.pdf?raw=true</x:v>
+      </x:c>
     </x:row>
     <x:row r="213">
       <x:c r="A213" t="str">
@@ -11919,6 +11928,12 @@
       <x:c r="U213" t="str"/>
       <x:c r="V213" t="str"/>
       <x:c r="W213" t="str"/>
+      <x:c r="X213" t="str">
+        <x:v>Urban Grey 099 / TEW Series=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/saman-SDS_Water-based-wood-stain.pdf?raw=true</x:v>
+      </x:c>
+      <x:c r="Z213" t="str">
+        <x:v>Urban Grey 099 / TEW Series=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/saman-TDS-ANG_TEW.pdf?raw=true</x:v>
+      </x:c>
     </x:row>
     <x:row r="214">
       <x:c r="A214" t="str">

</xml_diff>

<commit_message>
Add manufacturer SDS and TDS batch 099-101
</commit_message>
<xml_diff>
--- a/products_categories_descriptions_documents_working.xlsx
+++ b/products_categories_descriptions_documents_working.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" r:id="R1df7d6abc79948a7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" r:id="Ra1766d8c144e4abc"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -11983,6 +11983,12 @@
       <x:c r="U214" t="str"/>
       <x:c r="V214" t="str"/>
       <x:c r="W214" t="str"/>
+      <x:c r="X214" t="str">
+        <x:v>Dead Flat SAM-801=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/saman-SDS_SAM-801.pdf?raw=true</x:v>
+      </x:c>
+      <x:c r="Z214" t="str">
+        <x:v>Dead Flat SAM-801=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/saman-TDS-ANG_SAM-801.pdf?raw=true</x:v>
+      </x:c>
     </x:row>
     <x:row r="215">
       <x:c r="A215" t="str">
@@ -12036,6 +12042,12 @@
       <x:c r="U215" t="str"/>
       <x:c r="V215" t="str"/>
       <x:c r="W215" t="str"/>
+      <x:c r="X215" t="str">
+        <x:v>Flat / Satin / Semi-Gloss SAM-805 / SAM-830 / SAM-870=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/saman-SDS_SAM-805-SAM-830-and-SAM-870.pdf?raw=true</x:v>
+      </x:c>
+      <x:c r="Z215" t="str">
+        <x:v>Satin / Semi-Gloss SAM-830 / SAM-870=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/saman-TDS-ANG_SAM-830-870.pdf?raw=true</x:v>
+      </x:c>
     </x:row>
     <x:row r="216">
       <x:c r="A216" t="str">
@@ -12089,6 +12101,12 @@
       <x:c r="U216" t="str"/>
       <x:c r="V216" t="str"/>
       <x:c r="W216" t="str"/>
+      <x:c r="X216" t="str">
+        <x:v>Flat / Satin / Semi-Gloss / Gloss 160 Series=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/saman-SDS_160-005-160-031-160-051-160-091.pdf?raw=true</x:v>
+      </x:c>
+      <x:c r="Z216" t="str">
+        <x:v>Flat / Satin / Semi-Gloss / Gloss 160 Series=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/saman-TDS-ANG_varnish-160.pdf?raw=true</x:v>
+      </x:c>
     </x:row>
     <x:row r="217">
       <x:c r="A217" t="str">

</xml_diff>

<commit_message>
Add ZeraBrite SDS and TDS batch 102-104
</commit_message>
<xml_diff>
--- a/products_categories_descriptions_documents_working.xlsx
+++ b/products_categories_descriptions_documents_working.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" r:id="Ra1766d8c144e4abc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" r:id="R79680580cc6549c5"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -12401,6 +12401,12 @@
       <x:c r="U222" t="str"/>
       <x:c r="V222" t="str"/>
       <x:c r="W222" t="str"/>
+      <x:c r="X222" t="str">
+        <x:v>ZeraBrite CL-121 Parts A and B=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/zeraus-ZeraBrite_SD.pdf?raw=true</x:v>
+      </x:c>
+      <x:c r="Z222" t="str">
+        <x:v>ZeraBrite CL-121=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/zeraus-ZeraBrite_CL-121_tds.pdf?raw=true</x:v>
+      </x:c>
     </x:row>
     <x:row r="223">
       <x:c r="A223" t="str">

</xml_diff>

<commit_message>
Add ZeraDur and Insl-X documents batch 105-107
</commit_message>
<xml_diff>
--- a/products_categories_descriptions_documents_working.xlsx
+++ b/products_categories_descriptions_documents_working.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" r:id="R79680580cc6549c5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" r:id="Refc64ba7596c4121"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -12554,6 +12554,12 @@
       <x:c r="U225" t="str"/>
       <x:c r="V225" t="str"/>
       <x:c r="W225" t="str"/>
+      <x:c r="X225" t="str">
+        <x:v>ZeraDur 100 Parts A and B=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/zeraus-ZeraDur-100_SD.pdf?raw=true</x:v>
+      </x:c>
+      <x:c r="Z225" t="str">
+        <x:v>ZeraDur 100=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/zeraus-ZeraDur-100_TDS.pdf?raw=true</x:v>
+      </x:c>
     </x:row>
     <x:row r="226">
       <x:c r="A226" t="str">
@@ -14975,6 +14981,12 @@
       <x:c r="U276" t="str"/>
       <x:c r="V276" t="str"/>
       <x:c r="W276" t="str"/>
+      <x:c r="X276" t="str">
+        <x:v>Flat White FR-210=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/insl-x-FR-2100_SDS_EN.pdf?raw=true</x:v>
+      </x:c>
+      <x:c r="Z276" t="str">
+        <x:v>Flat White FR-210=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/insl-x-FR-210_TDS_EN.pdf?raw=true</x:v>
+      </x:c>
     </x:row>
     <x:row r="277">
       <x:c r="A277" t="str">

</xml_diff>

<commit_message>
Add Benjamin Moore HP documents batch 108-110
</commit_message>
<xml_diff>
--- a/products_categories_descriptions_documents_working.xlsx
+++ b/products_categories_descriptions_documents_working.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" r:id="Refc64ba7596c4121"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" r:id="R54d242ab55b14b82"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -15034,6 +15034,12 @@
       <x:c r="U277" t="str"/>
       <x:c r="V277" t="str"/>
       <x:c r="W277" t="str"/>
+      <x:c r="X277" t="str">
+        <x:v>HP1560-00FR Clear Sealer=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-HP1560-00FR_SDS_EN.pdf?raw=true|HP1560-90FR Catalyst=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-HP1560-90FR_SDS_EN.pdf?raw=true</x:v>
+      </x:c>
+      <x:c r="Z277" t="str">
+        <x:v>HP1560FR=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/benjamin-moore-HP1560_TDS_CE.pdf?raw=true</x:v>
+      </x:c>
     </x:row>
     <x:row r="278">
       <x:c r="A278" t="str">
@@ -15089,6 +15095,12 @@
       <x:c r="U278" t="str"/>
       <x:c r="V278" t="str"/>
       <x:c r="W278" t="str"/>
+      <x:c r="X278" t="str">
+        <x:v>HP2210-01FR White=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-HP2210-01FR_SDS_EN.pdf?raw=true|HP2210-7BFR Base=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-HP2210-7BFR_SDS_EN.pdf?raw=true|HP2210-80FR Black=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-HP2210-80FR_SDS_EN.pdf?raw=true|HP2210-8BFR Base=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-HP2210-8BFR_SDS_EN.pdf?raw=true|HP2210-9BFR Clear Base=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-HP2210-9BFR_SDS_EN.pdf?raw=true</x:v>
+      </x:c>
+      <x:c r="Z278" t="str">
+        <x:v>HP2210FR Semi-Gloss=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/benjamin-moore-HP2210_TDS_CE.pdf?raw=true</x:v>
+      </x:c>
     </x:row>
     <x:row r="279">
       <x:c r="A279" t="str">
@@ -15136,6 +15148,12 @@
       <x:c r="U279" t="str"/>
       <x:c r="V279" t="str"/>
       <x:c r="W279" t="str"/>
+      <x:c r="X279" t="str">
+        <x:v>HP2300-01FR White=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-HP2300-01FR_SDS_EN.pdf?raw=true</x:v>
+      </x:c>
+      <x:c r="Z279" t="str">
+        <x:v>HP2300FR Gloss=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/benjamin-moore-HP2300_TDS_CE.pdf?raw=true</x:v>
+      </x:c>
     </x:row>
     <x:row r="280">
       <x:c r="A280" t="str">

</xml_diff>

<commit_message>
Add Benjamin Moore coatings documents batch 111-113
</commit_message>
<xml_diff>
--- a/products_categories_descriptions_documents_working.xlsx
+++ b/products_categories_descriptions_documents_working.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" r:id="R54d242ab55b14b82"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" r:id="R083cde50f7474081"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -15201,6 +15201,12 @@
       <x:c r="U280" t="str"/>
       <x:c r="V280" t="str"/>
       <x:c r="W280" t="str"/>
+      <x:c r="X280" t="str">
+        <x:v>HP2400-7BFR=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-HP2400-7BFR_SDS_EN.pdf?raw=true|HP2400-10FR=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-HP2400-10FR_SDS_EN.pdf?raw=true|HP2400-80FR=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-HP2400-80FR_SDS_EN.pdf?raw=true|HP2400-9BFR=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-HP2400-9BFR_SDS_EN.pdf?raw=true|HP2400-8BFR=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-HP2400-8BFR_SDS_EN.pdf?raw=true</x:v>
+      </x:c>
+      <x:c r="Z280" t="str">
+        <x:v>HP2400FR Gloss=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/benjamin-moore-HP2400_TDS_CE.pdf?raw=true</x:v>
+      </x:c>
     </x:row>
     <x:row r="281">
       <x:c r="A281" t="str">
@@ -15248,6 +15254,12 @@
       <x:c r="U281" t="str"/>
       <x:c r="V281" t="str"/>
       <x:c r="W281" t="str"/>
+      <x:c r="X281" t="str">
+        <x:v>HP4400-00FR=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-HP4400-00FR_SDS_EN.pdf?raw=true|HP4400-7XFR=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-HP4400-7XFR_SDS_EN.pdf?raw=true|HP4400-8XFR=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-HP4400-8XFR_SDS_EN.pdf?raw=true|HP4400-9XFR=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-HP4400-9XFR_SDS_EN.pdf?raw=true|HP4400-70FR=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-HP4400-70FR_SDS_EN.pdf?raw=true|HP4400-75FR=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-HP4400-75FR_SDS_EN.pdf?raw=true|HP4400-90FR Catalyst=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-HP4400-90FR_SDS_EN.pdf?raw=true</x:v>
+      </x:c>
+      <x:c r="Z281" t="str">
+        <x:v>HP4400FR Gloss=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/benjamin-moore-HP4400_TDS_CE.pdf?raw=true</x:v>
+      </x:c>
     </x:row>
     <x:row r="282">
       <x:c r="A282" t="str">
@@ -15530,6 +15542,12 @@
       <x:c r="U287" t="str"/>
       <x:c r="V287" t="str"/>
       <x:c r="W287" t="str"/>
+      <x:c r="X287" t="str">
+        <x:v>K395-01=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-K39501_SDS_EN.pdf?raw=true|K395-1X=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-K3951X_SDS_EN.pdf?raw=true|K395-2X=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-K3952X_SDS_EN.pdf?raw=true|K395-80=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-K395380_SDS_EN.pdf?raw=true|K395-4X=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-K3954X_SDS_EN.pdf?raw=true|K395-3X=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-K3953X_SDS_EN.pdf?raw=true</x:v>
+      </x:c>
+      <x:c r="Z287" t="str">
+        <x:v>K395 Flat=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/benjamin-moore-K395_TDS_CE.pdf?raw=true</x:v>
+      </x:c>
     </x:row>
     <x:row r="288">
       <x:c r="A288" t="str">

</xml_diff>

<commit_message>
Add paint and primer documents batch 114-116
</commit_message>
<xml_diff>
--- a/products_categories_descriptions_documents_working.xlsx
+++ b/products_categories_descriptions_documents_working.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" r:id="R083cde50f7474081"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" r:id="R2fd656e4b5c04f3c"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -15642,6 +15642,12 @@
       <x:c r="U289" t="str"/>
       <x:c r="V289" t="str"/>
       <x:c r="W289" t="str"/>
+      <x:c r="X289" t="str">
+        <x:v>Knight Gray NSU-1007FR=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/insl-x-NSU-1007FR_SDS_EN.pdf?raw=true</x:v>
+      </x:c>
+      <x:c r="Z289" t="str">
+        <x:v>Sure Step NSU-10XXFR=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/insl-x-NSU-10XX_TDS_CAE.pdf?raw=true</x:v>
+      </x:c>
     </x:row>
     <x:row r="290">
       <x:c r="A290" t="str">
@@ -15689,6 +15695,12 @@
       <x:c r="U290" t="str"/>
       <x:c r="V290" t="str"/>
       <x:c r="W290" t="str"/>
+      <x:c r="X290" t="str">
+        <x:v>R13-1FR Semi-Gloss White=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/coronado-R13-1FR_SDS_EN.pdf?raw=true</x:v>
+      </x:c>
+      <x:c r="Z290" t="str">
+        <x:v>R13 Semi-Gloss=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/coronado-R13_TDS_US.pdf?raw=true</x:v>
+      </x:c>
     </x:row>
     <x:row r="291">
       <x:c r="A291" t="str">
@@ -15783,6 +15795,12 @@
       <x:c r="U292" t="str"/>
       <x:c r="V292" t="str"/>
       <x:c r="W292" t="str"/>
+      <x:c r="X292" t="str">
+        <x:v>K100-00 White=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-K10000_EN_SDS.pdf?raw=true|K100-04 Deep Base=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-K10004_MSDS_EN.pdf?raw=true</x:v>
+      </x:c>
+      <x:c r="Z292" t="str">
+        <x:v>K100 Exterior Wood Primer=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/benjamin-moore-20200110-K100-TDS-CE-OKF.pdf?raw=true</x:v>
+      </x:c>
     </x:row>
     <x:row r="293">
       <x:c r="A293" t="str">

</xml_diff>

<commit_message>
Add coating documents batch 117-119
</commit_message>
<xml_diff>
--- a/products_categories_descriptions_documents_working.xlsx
+++ b/products_categories_descriptions_documents_working.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" r:id="R2fd656e4b5c04f3c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" r:id="R844d0742bc8b454e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -15495,6 +15495,12 @@
       <x:c r="U286" t="str"/>
       <x:c r="V286" t="str"/>
       <x:c r="W286" t="str"/>
+      <x:c r="X286" t="str">
+        <x:v>K359-01 Flat White=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-K35901_SDS_EN.pdf?raw=true|K359-1X Base 1=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-K3591X_SDS_EN.pdf?raw=true|K359-2X Base 2=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-K3592X_SDS_EN.pdf?raw=true|K359-3X Base 3=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-K3593X_SDS_EN.pdf?raw=true|K359-4X Base 4=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/benjamin-moore-K3594X_SDS_EN.pdf?raw=true</x:v>
+      </x:c>
+      <x:c r="Z286" t="str">
+        <x:v>K359 Flat=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/benjamin-moore-K359_TDS_CE.pdf?raw=true</x:v>
+      </x:c>
     </x:row>
     <x:row r="287">
       <x:c r="A287" t="str">
@@ -15748,6 +15754,12 @@
       <x:c r="U291" t="str"/>
       <x:c r="V291" t="str"/>
       <x:c r="W291" t="str"/>
+      <x:c r="X291" t="str">
+        <x:v>TP-2210F White=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/insl-x-TP-2210F_SDS_EN.pdf?raw=true</x:v>
+      </x:c>
+      <x:c r="Z291" t="str">
+        <x:v>TP-22XXF Latex Traffic Paint=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/insl-x-TP-22XX_CAE.pdf?raw=true</x:v>
+      </x:c>
     </x:row>
     <x:row r="292">
       <x:c r="A292" t="str">
@@ -19139,6 +19151,12 @@
       <x:c r="U362" t="str"/>
       <x:c r="V362" t="str"/>
       <x:c r="W362" t="str"/>
+      <x:c r="X362" t="str">
+        <x:v>CUTEK Extreme Canada/US=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/cutek-CUTEK-Extreme-EN-Canada-US-SDS-2025-03-30-2.pdf?raw=true</x:v>
+      </x:c>
+      <x:c r="Z362" t="str">
+        <x:v>CUTEK Extreme Canada=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/cutek-CUTEK--Extreme-TDS-Canada-English-Web.pdf?raw=true</x:v>
+      </x:c>
     </x:row>
     <x:row r="363">
       <x:c r="A363" t="str">

</xml_diff>

<commit_message>
Add coating documents batch 120-122
</commit_message>
<xml_diff>
--- a/products_categories_descriptions_documents_working.xlsx
+++ b/products_categories_descriptions_documents_working.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" r:id="R844d0742bc8b454e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" r:id="R9d0e44a8ad2c4f0c"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -20403,6 +20403,12 @@
       <x:c r="U388" t="str"/>
       <x:c r="V388" t="str"/>
       <x:c r="W388" t="str"/>
+      <x:c r="Y388" t="str">
+        <x:v>TracSafe Anti-Slip Sealer=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/tracsafe-SDS-TracSafe-Anti-Slip-Sealer-ENG.pdf?raw=true</x:v>
+      </x:c>
+      <x:c r="Z388" t="str">
+        <x:v>TracSafe Anti-Slip Sealer Instruction Sheet=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/tracsafe-TracSafe-Anti-Slip-Sealer-Instructions.pdf?raw=true</x:v>
+      </x:c>
     </x:row>
     <x:row r="389">
       <x:c r="A389" t="str">
@@ -20497,6 +20503,12 @@
       <x:c r="U390" t="str"/>
       <x:c r="V390" t="str"/>
       <x:c r="W390" t="str"/>
+      <x:c r="Y390" t="str">
+        <x:v>Terrazzo Decorative Granite Coating=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/terrazzo-SDS-Terrazzo-Coating-ENG.pdf?raw=true</x:v>
+      </x:c>
+      <x:c r="Z390" t="str">
+        <x:v>Terrazzo Installation Instructions=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/terrazzo-Terrazzo-Installation-Instructions.pdf?raw=true</x:v>
+      </x:c>
     </x:row>
     <x:row r="391">
       <x:c r="A391" t="str">
@@ -21257,6 +21269,12 @@
       <x:c r="U406" t="str"/>
       <x:c r="V406" t="str"/>
       <x:c r="W406" t="str"/>
+      <x:c r="X406" t="str">
+        <x:v>Quick Coat Rosewood Quart 861390000=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/duraseal-Quick-Coat-Rosewood-861390000-SDS.pdf?raw=true</x:v>
+      </x:c>
+      <x:c r="Z406" t="str">
+        <x:v>Quick Coat Rosewood Quart 861390000 PDS=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/duraseal-Quick-Coat-861390000-PDS.pdf?raw=true</x:v>
+      </x:c>
     </x:row>
     <x:row r="407">
       <x:c r="A407" t="str">

</xml_diff>

<commit_message>
Add coating documents batch 123-125
</commit_message>
<xml_diff>
--- a/products_categories_descriptions_documents_working.xlsx
+++ b/products_categories_descriptions_documents_working.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" r:id="R9d0e44a8ad2c4f0c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" r:id="Rd0d1742c3e3d4a03"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -21377,6 +21377,12 @@
       <x:c r="U408" t="str"/>
       <x:c r="V408" t="str"/>
       <x:c r="W408" t="str"/>
+      <x:c r="Y408" t="str">
+        <x:v>985202-5P Federal Yellow=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/ennis-flint-985202-5P-Federal-Yellow-SDS.pdf?raw=true</x:v>
+      </x:c>
+      <x:c r="Z408" t="str">
+        <x:v>EF Series Fast Dry Waterborne 1952E/F Type I-II=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/ennis-flint-EF-Series-Fast-Dry-Waterborne-Traffic-Paint-PDS.pdf?raw=true</x:v>
+      </x:c>
     </x:row>
     <x:row r="409">
       <x:c r="A409" t="str">
@@ -21424,6 +21430,12 @@
       <x:c r="U409" t="str"/>
       <x:c r="V409" t="str"/>
       <x:c r="W409" t="str"/>
+      <x:c r="Y409" t="str">
+        <x:v>985201-5P Federal White=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/ennis-flint-985201-5P-Federal-White-SDS.pdf?raw=true</x:v>
+      </x:c>
+      <x:c r="Z409" t="str">
+        <x:v>EF Series Fast Dry Waterborne 1952E/F Type I-II=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/ennis-flint-EF-Series-Fast-Dry-Waterborne-Traffic-Paint-PDS.pdf?raw=true</x:v>
+      </x:c>
     </x:row>
     <x:row r="410">
       <x:c r="A410" t="str">
@@ -21565,6 +21577,12 @@
       <x:c r="U412" t="str"/>
       <x:c r="V412" t="str"/>
       <x:c r="W412" t="str"/>
+      <x:c r="Y412" t="str">
+        <x:v>985205-5P Handicap Blue=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/ennis-flint-985205-5P-Handicap-Blue-SDS.pdf?raw=true</x:v>
+      </x:c>
+      <x:c r="Z412" t="str">
+        <x:v>EF Series Fast Dry Waterborne 1952E/F Type I-II=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/ennis-flint-EF-Series-Fast-Dry-Waterborne-Traffic-Paint-PDS.pdf?raw=true</x:v>
+      </x:c>
     </x:row>
     <x:row r="413">
       <x:c r="A413" t="str">

</xml_diff>

<commit_message>
Add Krylon Fusion coating documents 126-129
</commit_message>
<xml_diff>
--- a/products_categories_descriptions_documents_working.xlsx
+++ b/products_categories_descriptions_documents_working.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" r:id="Rd0d1742c3e3d4a03"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" r:id="R8c4e8bbdb6ff4aee"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -25077,6 +25077,12 @@
       <x:c r="U486" t="str"/>
       <x:c r="V486" t="str"/>
       <x:c r="W486" t="str"/>
+      <x:c r="X486" t="str">
+        <x:v>Fusion All-In-One Satin Black K02732007=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/krylon-Fusion-All-In-One-Satin-Black-K02732007-SDS.pdf?raw=true</x:v>
+      </x:c>
+      <x:c r="Z486" t="str">
+        <x:v>Fusion All-In-One Satin Black K02732007=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/krylon-Fusion-All-In-One-Satin-Black-K02732007-PDS.pdf?raw=true</x:v>
+      </x:c>
     </x:row>
     <x:row r="487">
       <x:c r="A487" t="str">
@@ -25124,6 +25130,9 @@
       <x:c r="U487" t="str"/>
       <x:c r="V487" t="str"/>
       <x:c r="W487" t="str"/>
+      <x:c r="X487" t="str">
+        <x:v>Fusion All-In-One Metallic Gold K02770007=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/krylon-Fusion-All-In-One-Metallic-Gold-K02770007-SDS.pdf?raw=true</x:v>
+      </x:c>
     </x:row>
     <x:row r="488">
       <x:c r="A488" t="str">
@@ -25171,6 +25180,12 @@
       <x:c r="U488" t="str"/>
       <x:c r="V488" t="str"/>
       <x:c r="W488" t="str"/>
+      <x:c r="X488" t="str">
+        <x:v>Fusion All-In-One Gloss Black K02702007=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/krylon-Fusion-All-In-One-Gloss-Black-K02702007-SDS.pdf?raw=true</x:v>
+      </x:c>
+      <x:c r="Z488" t="str">
+        <x:v>Fusion All-In-One Gloss Black K02702007=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/krylon-Fusion-All-In-One-Gloss-Black-K02702007-PDS.pdf?raw=true</x:v>
+      </x:c>
     </x:row>
     <x:row r="489">
       <x:c r="A489" t="str">
@@ -25218,6 +25233,12 @@
       <x:c r="U489" t="str"/>
       <x:c r="V489" t="str"/>
       <x:c r="W489" t="str"/>
+      <x:c r="X489" t="str">
+        <x:v>Fusion All-In-One Flat Black K02728007=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/krylon-Fusion-All-In-One-Flat-Black-K02728007-SDS.pdf?raw=true</x:v>
+      </x:c>
+      <x:c r="Z489" t="str">
+        <x:v>Fusion All-In-One Flat Black K02728007=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/krylon-Fusion-All-In-One-Flat-Black-K02728007-PDS.pdf?raw=true</x:v>
+      </x:c>
     </x:row>
     <x:row r="490">
       <x:c r="A490" t="str">

</xml_diff>

<commit_message>
Add wood finish documents 130-132
</commit_message>
<xml_diff>
--- a/products_categories_descriptions_documents_working.xlsx
+++ b/products_categories_descriptions_documents_working.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" r:id="R8c4e8bbdb6ff4aee"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" r:id="R494b3cb380374225"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -25286,6 +25286,12 @@
       <x:c r="U490" t="str"/>
       <x:c r="V490" t="str"/>
       <x:c r="W490" t="str"/>
+      <x:c r="X490" t="str">
+        <x:v>Marine &amp; Door Oil Spar Varnish Satin 50801/50804=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/last-n-last-Marine-Door-Oil-Spar-Varnish-Satin-50801-50804-SDS.pdf?raw=true</x:v>
+      </x:c>
+      <x:c r="Z490" t="str">
+        <x:v>Marine &amp; Door Oil Spar Varnish 50701-50804=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/last-n-last-Marine-Door-Oil-Spar-Varnish-50701-50804-TDS.pdf?raw=true</x:v>
+      </x:c>
     </x:row>
     <x:row r="491">
       <x:c r="A491" t="str">
@@ -25333,6 +25339,9 @@
       <x:c r="U491" t="str"/>
       <x:c r="V491" t="str"/>
       <x:c r="W491" t="str"/>
+      <x:c r="X491" t="str">
+        <x:v>Clear Polyurethane Wood Finish Gloss 350 VOC 53501=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/last-n-last-Clear-Polyurethane-Wood-Finish-Gloss-350-VOC-53501-SDS.pdf?raw=true</x:v>
+      </x:c>
     </x:row>
     <x:row r="492">
       <x:c r="A492" t="str">
@@ -25380,6 +25389,9 @@
       <x:c r="U492" t="str"/>
       <x:c r="V492" t="str"/>
       <x:c r="W492" t="str"/>
+      <x:c r="X492" t="str">
+        <x:v>Professional Polyurethane Satin 350 VOC 89511/89512/89515=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/last-n-last-Professional-Polyurethane-Satin-350-VOC-89511-89512-89515-SDS.pdf?raw=true</x:v>
+      </x:c>
     </x:row>
     <x:row r="493">
       <x:c r="A493" t="str">

</xml_diff>

<commit_message>
Add primer and decorative coating documents 133-136
</commit_message>
<xml_diff>
--- a/products_categories_descriptions_documents_working.xlsx
+++ b/products_categories_descriptions_documents_working.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" r:id="R494b3cb380374225"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" r:id="R31d5038bec944ed7"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -25823,6 +25823,9 @@
       <x:c r="U501" t="str"/>
       <x:c r="V501" t="str"/>
       <x:c r="W501" t="str"/>
+      <x:c r="Y501" t="str">
+        <x:v>KILZ Original Low Odor Interior Primer Aerosol 1044=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/kilz-Original-Low-Odor-Interior-Primer-Aerosol-1044-SDS.pdf?raw=true</x:v>
+      </x:c>
     </x:row>
     <x:row r="502">
       <x:c r="A502" t="str">
@@ -25870,6 +25873,12 @@
       <x:c r="U502" t="str"/>
       <x:c r="V502" t="str"/>
       <x:c r="W502" t="str"/>
+      <x:c r="X502" t="str">
+        <x:v>Tonachino Firenze=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/meoded-Tonachino-Firenze-SDS.pdf?raw=true</x:v>
+      </x:c>
+      <x:c r="Z502" t="str">
+        <x:v>Tonachino Firenze=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/meoded-Tonachino-Firenze-TDS.pdf?raw=true</x:v>
+      </x:c>
     </x:row>
     <x:row r="503">
       <x:c r="A503" t="str">
@@ -25917,6 +25926,12 @@
       <x:c r="U503" t="str"/>
       <x:c r="V503" t="str"/>
       <x:c r="W503" t="str"/>
+      <x:c r="X503" t="str">
+        <x:v>Stucco Lamundo=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/meoded-Stucco-Lamundo-SDS.pdf?raw=true</x:v>
+      </x:c>
+      <x:c r="Z503" t="str">
+        <x:v>Stucco Lamundo=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/meoded-Stucco-Lamundo-TDS.pdf?raw=true</x:v>
+      </x:c>
     </x:row>
     <x:row r="504">
       <x:c r="A504" t="str">
@@ -25964,6 +25979,12 @@
       <x:c r="U504" t="str"/>
       <x:c r="V504" t="str"/>
       <x:c r="W504" t="str"/>
+      <x:c r="X504" t="str">
+        <x:v>Stain Shield Sealer=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/meoded-Stain-Shield-Sealer-SDS.pdf?raw=true</x:v>
+      </x:c>
+      <x:c r="Z504" t="str">
+        <x:v>Stain Shield Sealer=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/meoded-Stain-Shield-Sealer-TDS.pdf?raw=true</x:v>
+      </x:c>
     </x:row>
     <x:row r="505">
       <x:c r="A505" t="str">

</xml_diff>

<commit_message>
Add Meoded coating documents 137-148
</commit_message>
<xml_diff>
--- a/products_categories_descriptions_documents_working.xlsx
+++ b/products_categories_descriptions_documents_working.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" r:id="R31d5038bec944ed7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" r:id="R1b3e473334ef4b75"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -26032,6 +26032,12 @@
       <x:c r="U505" t="str"/>
       <x:c r="V505" t="str"/>
       <x:c r="W505" t="str"/>
+      <x:c r="X505" t="str">
+        <x:v>PlasterSeal Plus Part A=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/meoded-PlasterSeal-Plus-Part-A-SDS.pdf?raw=true|PlasterSeal Plus Part B=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/meoded-PlasterSeal-Plus-Part-B-SDS.pdf?raw=true</x:v>
+      </x:c>
+      <x:c r="Z505" t="str">
+        <x:v>PlasterSeal Plus System=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/meoded-PlasterSeal-Plus-System-TDS.pdf?raw=true</x:v>
+      </x:c>
     </x:row>
     <x:row r="506">
       <x:c r="A506" t="str">
@@ -26087,6 +26093,12 @@
       <x:c r="U506" t="str"/>
       <x:c r="V506" t="str"/>
       <x:c r="W506" t="str"/>
+      <x:c r="X506" t="str">
+        <x:v>PlasterGuard Sealer=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/meoded-PlasterGuard-Sealer-SDS.pdf?raw=true</x:v>
+      </x:c>
+      <x:c r="Z506" t="str">
+        <x:v>PlasterGuard Sealer=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/meoded-PlasterGuard-Sealer-TDS.pdf?raw=true</x:v>
+      </x:c>
     </x:row>
     <x:row r="507">
       <x:c r="A507" t="str">
@@ -26134,6 +26146,12 @@
       <x:c r="U507" t="str"/>
       <x:c r="V507" t="str"/>
       <x:c r="W507" t="str"/>
+      <x:c r="X507" t="str">
+        <x:v>Pearlas Velvet=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/meoded-Pearlas-Velvet-SDS.pdf?raw=true</x:v>
+      </x:c>
+      <x:c r="Z507" t="str">
+        <x:v>Pearlas Velvet=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/meoded-Pearlas-Velvet-TDS.pdf?raw=true</x:v>
+      </x:c>
     </x:row>
     <x:row r="508">
       <x:c r="A508" t="str">
@@ -26181,6 +26199,12 @@
       <x:c r="U508" t="str"/>
       <x:c r="V508" t="str"/>
       <x:c r="W508" t="str"/>
+      <x:c r="X508" t="str">
+        <x:v>Quartz Primer=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/meoded-Quartz-Primer-SDS.pdf?raw=true</x:v>
+      </x:c>
+      <x:c r="Z508" t="str">
+        <x:v>Quartz Primer=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/meoded-Quartz-Primer-TDS.pdf?raw=true</x:v>
+      </x:c>
     </x:row>
     <x:row r="509">
       <x:c r="A509" t="str">
@@ -26228,6 +26252,12 @@
       <x:c r="U509" t="str"/>
       <x:c r="V509" t="str"/>
       <x:c r="W509" t="str"/>
+      <x:c r="X509" t="str">
+        <x:v>Moroccan Clay=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/meoded-Moroccan-Clay-SDS.pdf?raw=true</x:v>
+      </x:c>
+      <x:c r="Z509" t="str">
+        <x:v>Moroccan Clay=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/meoded-Moroccan-Clay-TDS.pdf?raw=true</x:v>
+      </x:c>
     </x:row>
     <x:row r="510">
       <x:c r="A510" t="str">
@@ -26275,6 +26305,12 @@
       <x:c r="U510" t="str"/>
       <x:c r="V510" t="str"/>
       <x:c r="W510" t="str"/>
+      <x:c r="X510" t="str">
+        <x:v>Lime Wash=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/meoded-Lime-Wash-SDS.pdf?raw=true</x:v>
+      </x:c>
+      <x:c r="Z510" t="str">
+        <x:v>Lime Wash=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/meoded-Lime-Wash-TDS.pdf?raw=true</x:v>
+      </x:c>
     </x:row>
     <x:row r="511">
       <x:c r="A511" t="str">
@@ -26322,6 +26358,12 @@
       <x:c r="U511" t="str"/>
       <x:c r="V511" t="str"/>
       <x:c r="W511" t="str"/>
+      <x:c r="X511" t="str">
+        <x:v>Marmorino Palladino=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/meoded-Marmorino-Palladino-SDS.pdf?raw=true</x:v>
+      </x:c>
+      <x:c r="Z511" t="str">
+        <x:v>Marmorino Palladino=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/meoded-Marmorino-Palladino-TDS.pdf?raw=true</x:v>
+      </x:c>
     </x:row>
     <x:row r="512">
       <x:c r="A512" t="str">
@@ -26416,6 +26458,12 @@
       <x:c r="U513" t="str"/>
       <x:c r="V513" t="str"/>
       <x:c r="W513" t="str"/>
+      <x:c r="X513" t="str">
+        <x:v>Hydrowax=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/meoded-Hydrowax-SDS.pdf?raw=true</x:v>
+      </x:c>
+      <x:c r="Z513" t="str">
+        <x:v>Hydrowax=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/meoded-Hydrowax-TDS.pdf?raw=true</x:v>
+      </x:c>
     </x:row>
     <x:row r="514">
       <x:c r="A514" t="str">
@@ -26463,6 +26511,12 @@
       <x:c r="U514" t="str"/>
       <x:c r="V514" t="str"/>
       <x:c r="W514" t="str"/>
+      <x:c r="X514" t="str">
+        <x:v>Golmex=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/meoded-Golmex-SDS.pdf?raw=true</x:v>
+      </x:c>
+      <x:c r="Z514" t="str">
+        <x:v>Golmex=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/meoded-Golmex-TDS.pdf?raw=true</x:v>
+      </x:c>
     </x:row>
     <x:row r="515">
       <x:c r="A515" t="str">
@@ -26510,6 +26564,12 @@
       <x:c r="U515" t="str"/>
       <x:c r="V515" t="str"/>
       <x:c r="W515" t="str"/>
+      <x:c r="X515" t="str">
+        <x:v>Crystal Brush Glitter Paint=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/meoded-Crystal-Brush-Glitter-Paint-SDS.pdf?raw=true</x:v>
+      </x:c>
+      <x:c r="Z515" t="str">
+        <x:v>Crystal Brush Glitter Paint=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/meoded-Crystal-Brush-Glitter-Paint-TDS.pdf?raw=true</x:v>
+      </x:c>
     </x:row>
     <x:row r="516">
       <x:c r="A516" t="str">
@@ -26557,6 +26617,12 @@
       <x:c r="U516" t="str"/>
       <x:c r="V516" t="str"/>
       <x:c r="W516" t="str"/>
+      <x:c r="X516" t="str">
+        <x:v>Cristallo Clear=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/meoded-Cristallo-Clear-SDS.pdf?raw=true</x:v>
+      </x:c>
+      <x:c r="Z516" t="str">
+        <x:v>Cristallo Clear=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/meoded-Cristallo-Clear-TDS.pdf?raw=true</x:v>
+      </x:c>
     </x:row>
     <x:row r="517">
       <x:c r="A517" t="str">
@@ -26604,6 +26670,12 @@
       <x:c r="U517" t="str"/>
       <x:c r="V517" t="str"/>
       <x:c r="W517" t="str"/>
+      <x:c r="X517" t="str">
+        <x:v>Concretta FS=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/meoded-Concretta-FS-SDS.pdf?raw=true</x:v>
+      </x:c>
+      <x:c r="Z517" t="str">
+        <x:v>Concretta FS=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/meoded-Concretta-FS-TDS.pdf?raw=true</x:v>
+      </x:c>
     </x:row>
     <x:row r="518">
       <x:c r="A518" t="str">

</xml_diff>

<commit_message>
Add coating documents 149-158
</commit_message>
<xml_diff>
--- a/products_categories_descriptions_documents_working.xlsx
+++ b/products_categories_descriptions_documents_working.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" r:id="R1b3e473334ef4b75"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" r:id="R5566f5c4b6b74595"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -26723,6 +26723,12 @@
       <x:c r="U518" t="str"/>
       <x:c r="V518" t="str"/>
       <x:c r="W518" t="str"/>
+      <x:c r="X518" t="str">
+        <x:v>Messmer's UV Plus Natural - Standard/Federal VOC=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/messmer-s-Messmers-UV-Plus-Natural-Standard-SDS.pdf?raw=true</x:v>
+      </x:c>
+      <x:c r="Z518" t="str">
+        <x:v>Messmer's UV Plus=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/messmer-s-Messmers-UV-Plus-TDS.pdf?raw=true</x:v>
+      </x:c>
     </x:row>
     <x:row r="519">
       <x:c r="A519" t="str">
@@ -27060,6 +27066,12 @@
       <x:c r="U525" t="str"/>
       <x:c r="V525" t="str"/>
       <x:c r="W525" t="str"/>
+      <x:c r="X525" t="str">
+        <x:v>Minwax Wipe-On Poly Clear Gloss Quart=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/minwax-Minwax-Wipe-On-Poly-Clear-Gloss-Quart-SDS.pdf?raw=true|Minwax Wipe-On Poly Clear Satin Quart=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/minwax-Minwax-Wipe-On-Poly-Clear-Satin-Quart-SDS.pdf?raw=true</x:v>
+      </x:c>
+      <x:c r="Z525" t="str">
+        <x:v>Minwax Wipe-On Poly Clear Gloss=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/minwax-Minwax-Wipe-On-Poly-Clear-Gloss-PDS.pdf?raw=true|Minwax Wipe-On Poly Clear Satin=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/minwax-Minwax-Wipe-On-Poly-Clear-Satin-PDS.pdf?raw=true</x:v>
+      </x:c>
     </x:row>
     <x:row r="526">
       <x:c r="A526" t="str">
@@ -27107,6 +27119,12 @@
       <x:c r="U526" t="str"/>
       <x:c r="V526" t="str"/>
       <x:c r="W526" t="str"/>
+      <x:c r="X526" t="str">
+        <x:v>Minwax Tung Oil Finish Pint=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/minwax-Minwax-Tung-Oil-Finish-Pint-SDS.pdf?raw=true</x:v>
+      </x:c>
+      <x:c r="Z526" t="str">
+        <x:v>Minwax Tung Oil Finish=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/minwax-Minwax-Tung-Oil-Finish-PDS.pdf?raw=true</x:v>
+      </x:c>
     </x:row>
     <x:row r="527">
       <x:c r="A527" t="str">
@@ -27154,6 +27172,9 @@
       <x:c r="U527" t="str"/>
       <x:c r="V527" t="str"/>
       <x:c r="W527" t="str"/>
+      <x:c r="X527" t="str">
+        <x:v>Minwax Helmsman Teak Oil Quart=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/minwax-Minwax-Helmsman-Teak-Oil-Quart-SDS.pdf?raw=true</x:v>
+      </x:c>
     </x:row>
     <x:row r="528">
       <x:c r="A528" t="str">
@@ -27248,6 +27269,12 @@
       <x:c r="U529" t="str"/>
       <x:c r="V529" t="str"/>
       <x:c r="W529" t="str"/>
+      <x:c r="X529" t="str">
+        <x:v>Minwax Paste Finishing Wax Natural=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/minwax-Minwax-Paste-Finishing-Wax-Natural-SDS.pdf?raw=true</x:v>
+      </x:c>
+      <x:c r="Z529" t="str">
+        <x:v>Minwax Paste Finishing Wax Natural=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/minwax-Minwax-Paste-Finishing-Wax-Natural-PDS.pdf?raw=true</x:v>
+      </x:c>
     </x:row>
     <x:row r="530">
       <x:c r="A530" t="str">
@@ -27295,6 +27322,12 @@
       <x:c r="U530" t="str"/>
       <x:c r="V530" t="str"/>
       <x:c r="W530" t="str"/>
+      <x:c r="X530" t="str">
+        <x:v>Minwax Wood Finish Golden Oak 210B Quart=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/minwax-Minwax-Wood-Finish-Golden-Oak-210B-Quart-SDS.pdf?raw=true</x:v>
+      </x:c>
+      <x:c r="Z530" t="str">
+        <x:v>Minwax Wood Finish Golden Oak 210B=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/minwax-Minwax-Wood-Finish-Golden-Oak-210B-PDS.pdf?raw=true</x:v>
+      </x:c>
     </x:row>
     <x:row r="531">
       <x:c r="A531" t="str">
@@ -27389,6 +27422,12 @@
       <x:c r="U532" t="str"/>
       <x:c r="V532" t="str"/>
       <x:c r="W532" t="str"/>
+      <x:c r="X532" t="str">
+        <x:v>Minwax Oil-Based Pre-Stain Wood Conditioner Quart=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/minwax-Minwax-Oil-Based-Pre-Stain-Wood-Conditioner-Quart-SDS.pdf?raw=true</x:v>
+      </x:c>
+      <x:c r="Z532" t="str">
+        <x:v>Minwax Oil-Based Pre-Stain Wood Conditioner=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/minwax-Minwax-Oil-Based-Pre-Stain-Wood-Conditioner-PDS.pdf?raw=true</x:v>
+      </x:c>
     </x:row>
     <x:row r="533">
       <x:c r="A533" t="str">
@@ -27444,6 +27483,12 @@
       </x:c>
       <x:c r="V533" t="str"/>
       <x:c r="W533" t="str"/>
+      <x:c r="X533" t="str">
+        <x:v>Modern Masters Metallic Paint Flash Gold ME16406 6 oz=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/modern-masters-Modern-Masters-Metallic-Paint-Flash-Gold-ME16406-SDS.pdf?raw=true</x:v>
+      </x:c>
+      <x:c r="Z533" t="str">
+        <x:v>Modern Masters Metallic Paint Collection Satin=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/modern-masters-Modern-Masters-Metallic-Paint-Collection-Satin-TDS.pdf?raw=true</x:v>
+      </x:c>
     </x:row>
     <x:row r="534">
       <x:c r="A534" t="str">
@@ -27491,6 +27536,12 @@
       <x:c r="U534" t="str"/>
       <x:c r="V534" t="str"/>
       <x:c r="W534" t="str"/>
+      <x:c r="X534" t="str">
+        <x:v>Modern Masters MasterClear Supreme Satin MCS902GAL=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/modern-masters-Modern-Masters-MasterClear-Supreme-Satin-MCS902GAL-SDS.pdf?raw=true</x:v>
+      </x:c>
+      <x:c r="Z534" t="str">
+        <x:v>Modern Masters MasterClear Supreme=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/modern-masters-Modern-Masters-MasterClear-Supreme-TDS.pdf?raw=true</x:v>
+      </x:c>
     </x:row>
     <x:row r="535">
       <x:c r="A535" t="str">
@@ -27585,6 +27636,12 @@
       <x:c r="U536" t="str"/>
       <x:c r="V536" t="str"/>
       <x:c r="W536" t="str"/>
+      <x:c r="Y536" t="str">
+        <x:v>Klenk's Epoxy Enamel Gloss White 815201=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/klenk-s-Klenks-Epoxy-Enamel-Gloss-White-815201-SDS.pdf?raw=true</x:v>
+      </x:c>
+      <x:c r="Z536" t="str">
+        <x:v>Klenk's Epoxy Enamel=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/klenk-s-Klenks-Epoxy-Enamel-Directions-TDS.pdf?raw=true</x:v>
+      </x:c>
     </x:row>
     <x:row r="537">
       <x:c r="A537" t="str">

</xml_diff>

<commit_message>
Add wood coating documents 159-164
</commit_message>
<xml_diff>
--- a/products_categories_descriptions_documents_working.xlsx
+++ b/products_categories_descriptions_documents_working.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" r:id="R5566f5c4b6b74595"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" r:id="R73eb5fa19f3f4c1b"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -28723,6 +28723,12 @@
       <x:c r="U559" t="str"/>
       <x:c r="V559" t="str"/>
       <x:c r="W559" t="str"/>
+      <x:c r="X559" t="str">
+        <x:v>Solvable Boiled Linseed Oil 53-404=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/recochem-Solvable-Boiled-Linseed-Oil-53-404-SDS.pdf?raw=true</x:v>
+      </x:c>
+      <x:c r="Z559" t="str">
+        <x:v>Solvable Boiled Linseed Oil=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/recochem-Solvable-Boiled-Linseed-Oil-Application-Brochure-TDS.pdf?raw=true</x:v>
+      </x:c>
     </x:row>
     <x:row r="560">
       <x:c r="A560" t="str">
@@ -28770,6 +28776,12 @@
       <x:c r="U560" t="str"/>
       <x:c r="V560" t="str"/>
       <x:c r="W560" t="str"/>
+      <x:c r="X560" t="str">
+        <x:v>Penofin Ultra Premium Red Label Sable - 550 VOC=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/penofin-Penofin-Ultra-Premium-Red-Label-Sable-550-VOC-SDS.pdf?raw=true</x:v>
+      </x:c>
+      <x:c r="Z560" t="str">
+        <x:v>Penofin Ultra Premium Red Label=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/penofin-Penofin-Ultra-Premium-Red-Label-TDS.pdf?raw=true</x:v>
+      </x:c>
     </x:row>
     <x:row r="561">
       <x:c r="A561" t="str">
@@ -28817,6 +28829,12 @@
       <x:c r="U561" t="str"/>
       <x:c r="V561" t="str"/>
       <x:c r="W561" t="str"/>
+      <x:c r="X561" t="str">
+        <x:v>Penofin Architectural Grade TSF Hardwood - Natural=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/penofin-Penofin-Architectural-Grade-TSF-Hardwood-Natural-SDS.pdf?raw=true|Penofin Architectural Grade TSF Hardwood - Ipe=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/penofin-Penofin-Architectural-Grade-TSF-Hardwood-Ipe-SDS.pdf?raw=true</x:v>
+      </x:c>
+      <x:c r="Z561" t="str">
+        <x:v>Penofin Architectural Grade TSF Hardwood=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/penofin-Penofin-Architectural-Grade-TSF-Hardwood-TDS.pdf?raw=true</x:v>
+      </x:c>
     </x:row>
     <x:row r="562">
       <x:c r="A562" t="str">
@@ -28872,6 +28890,12 @@
       </x:c>
       <x:c r="V562" t="str"/>
       <x:c r="W562" t="str"/>
+      <x:c r="X562" t="str">
+        <x:v>Penofin Exterior Hardwood Formula - 550 VOC=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/penofin-Penofin-Exterior-Hardwood-Formula-550-VOC-SDS.pdf?raw=true</x:v>
+      </x:c>
+      <x:c r="Z562" t="str">
+        <x:v>Penofin Exterior Hardwood Formula=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/penofin-Penofin-Exterior-Hardwood-Formula-TDS.pdf?raw=true</x:v>
+      </x:c>
     </x:row>
     <x:row r="563">
       <x:c r="A563" t="str">
@@ -29742,6 +29766,12 @@
       <x:c r="U580" t="str"/>
       <x:c r="V580" t="str"/>
       <x:c r="W580" t="str"/>
+      <x:c r="X580" t="str">
+        <x:v>Olympic Rescue It Moderate Restoration 79705 Five Gallon=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/olympic-Olympic-Rescue-It-Moderate-Restoration-79705-Five-Gallon-SDS.pdf?raw=true</x:v>
+      </x:c>
+      <x:c r="Z580" t="str">
+        <x:v>Olympic Rescue It Moderate Restoration 79705 Five Gallon=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/olympic-Olympic-Rescue-It-Moderate-Restoration-79705-Five-Gallon-TDS.pdf?raw=true</x:v>
+      </x:c>
     </x:row>
     <x:row r="581">
       <x:c r="A581" t="str">
@@ -29789,6 +29819,12 @@
       <x:c r="U581" t="str"/>
       <x:c r="V581" t="str"/>
       <x:c r="W581" t="str"/>
+      <x:c r="X581" t="str">
+        <x:v>Olympic Maximum Semi-Transparent Neutral Base 79560C Five Gallon=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/olympic-Olympic-Maximum-Semi-Transparent-Neutral-79560C-Five-Gallon-SDS.pdf?raw=true</x:v>
+      </x:c>
+      <x:c r="Z581" t="str">
+        <x:v>Olympic Maximum Semi-Transparent Neutral Base 79560C Five Gallon=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/olympic-Olympic-Maximum-Semi-Transparent-Neutral-79560C-Five-Gallon-TDS.pdf?raw=true</x:v>
+      </x:c>
     </x:row>
     <x:row r="582">
       <x:c r="A582" t="str">

</xml_diff>

<commit_message>
Add ProTek coating documents 165-176
</commit_message>
<xml_diff>
--- a/products_categories_descriptions_documents_working.xlsx
+++ b/products_categories_descriptions_documents_working.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" r:id="R73eb5fa19f3f4c1b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" r:id="R2972247848a24863"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -31737,6 +31737,12 @@
       <x:c r="U621" t="str"/>
       <x:c r="V621" t="str"/>
       <x:c r="W621" t="str"/>
+      <x:c r="X621" t="str">
+        <x:v>ProTek Zero Gloss Varnish=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/protek-ProTek-Zero-Gloss-Varnish-SDS.pdf?raw=true</x:v>
+      </x:c>
+      <x:c r="Z621" t="str">
+        <x:v>ProTek Zero Gloss Varnish=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/protek-ProTek-Zero-Gloss-Varnish-Application-TDS.pdf?raw=true</x:v>
+      </x:c>
     </x:row>
     <x:row r="622">
       <x:c r="A622" t="str">
@@ -31784,6 +31790,12 @@
       <x:c r="U622" t="str"/>
       <x:c r="V622" t="str"/>
       <x:c r="W622" t="str"/>
+      <x:c r="X622" t="str">
+        <x:v>ProTek Texturtop Flat Wax Topcoat=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/textureline-ProTek-Texturtop-Flat-Wax-Topcoat-SDS.pdf?raw=true</x:v>
+      </x:c>
+      <x:c r="Z622" t="str">
+        <x:v>ProTek Flat Wax - Acrylic Venetian Plaster System=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/textureline-ProTek-Acrylic-Venetian-Plaster-System-TDS.pdf?raw=true</x:v>
+      </x:c>
     </x:row>
     <x:row r="623">
       <x:c r="A623" t="str">
@@ -31831,6 +31843,12 @@
       <x:c r="U623" t="str"/>
       <x:c r="V623" t="str"/>
       <x:c r="W623" t="str"/>
+      <x:c r="X623" t="str">
+        <x:v>ProTek Texturbase White=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/textureline-ProTek-Texturbase-White-SDS.pdf?raw=true|ProTek Texturbase Neutral=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/textureline-ProTek-Texturbase-Neutral-SDS.pdf?raw=true</x:v>
+      </x:c>
+      <x:c r="Z623" t="str">
+        <x:v>ProTek Acrylic Venetian Plaster=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/textureline-ProTek-Acrylic-Venetian-Plaster-System-TDS.pdf?raw=true</x:v>
+      </x:c>
     </x:row>
     <x:row r="624">
       <x:c r="A624" t="str">
@@ -31878,6 +31896,12 @@
       <x:c r="U624" t="str"/>
       <x:c r="V624" t="str"/>
       <x:c r="W624" t="str"/>
+      <x:c r="X624" t="str">
+        <x:v>ProTek Metaltech Silver T-27301 to T-27304=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/textureline-ProTek-Metaltech-Silver-SDS.pdf?raw=true</x:v>
+      </x:c>
+      <x:c r="Z624" t="str">
+        <x:v>ProTek Metaltech Metallic=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/textureline-ProTek-Metaltech-Metallic-TDS.pdf?raw=true</x:v>
+      </x:c>
     </x:row>
     <x:row r="625">
       <x:c r="A625" t="str">
@@ -31925,6 +31949,12 @@
       <x:c r="U625" t="str"/>
       <x:c r="V625" t="str"/>
       <x:c r="W625" t="str"/>
+      <x:c r="X625" t="str">
+        <x:v>ProTek Metaltech Pearl T-27001 to T-27004=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/textureline-ProTek-Metaltech-Pearl-SDS.pdf?raw=true</x:v>
+      </x:c>
+      <x:c r="Z625" t="str">
+        <x:v>ProTek Metaltech Metallic=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/textureline-ProTek-Metaltech-Metallic-TDS.pdf?raw=true</x:v>
+      </x:c>
     </x:row>
     <x:row r="626">
       <x:c r="A626" t="str">
@@ -31972,6 +32002,12 @@
       <x:c r="U626" t="str"/>
       <x:c r="V626" t="str"/>
       <x:c r="W626" t="str"/>
+      <x:c r="X626" t="str">
+        <x:v>ProTek Metaltech Gold T-27251 to T-27254=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/textureline-ProTek-Metaltech-Gold-SDS.pdf?raw=true</x:v>
+      </x:c>
+      <x:c r="Z626" t="str">
+        <x:v>ProTek Metaltech Metallic=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/textureline-ProTek-Metaltech-Metallic-TDS.pdf?raw=true</x:v>
+      </x:c>
     </x:row>
     <x:row r="627">
       <x:c r="A627" t="str">
@@ -32019,6 +32055,12 @@
       <x:c r="U627" t="str"/>
       <x:c r="V627" t="str"/>
       <x:c r="W627" t="str"/>
+      <x:c r="X627" t="str">
+        <x:v>ProTek Marmorino Classico=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/textureline-ProTek-Marmorino-Classico-SDS.pdf?raw=true</x:v>
+      </x:c>
+      <x:c r="Z627" t="str">
+        <x:v>ProTek Marmorino Classico Venetian Plaster=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/textureline-ProTek-Marmorino-Classico-Venetian-Plaster-TDS.pdf?raw=true</x:v>
+      </x:c>
     </x:row>
     <x:row r="628">
       <x:c r="A628" t="str">
@@ -32066,6 +32108,12 @@
       <x:c r="U628" t="str"/>
       <x:c r="V628" t="str"/>
       <x:c r="W628" t="str"/>
+      <x:c r="X628" t="str">
+        <x:v>ProTek Carolina Sandstone Spatula=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/textureline-ProTek-Carolina-Sandstone-SDS.pdf?raw=true</x:v>
+      </x:c>
+      <x:c r="Z628" t="str">
+        <x:v>ProTek Carolina Sandstone Acrylic Plaster=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/textureline-ProTek-Carolina-Sandstone-Acrylic-Plaster-TDS.pdf?raw=true</x:v>
+      </x:c>
     </x:row>
     <x:row r="629">
       <x:c r="A629" t="str">
@@ -32113,6 +32161,9 @@
       <x:c r="U629" t="str"/>
       <x:c r="V629" t="str"/>
       <x:c r="W629" t="str"/>
+      <x:c r="Z629" t="str">
+        <x:v>ProTek Burnishing Wax - Acrylic Venetian Plaster System=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/textureline-ProTek-Acrylic-Venetian-Plaster-System-TDS.pdf?raw=true</x:v>
+      </x:c>
     </x:row>
     <x:row r="630">
       <x:c r="A630" t="str">
@@ -32160,6 +32211,12 @@
       <x:c r="U630" t="str"/>
       <x:c r="V630" t="str"/>
       <x:c r="W630" t="str"/>
+      <x:c r="X630" t="str">
+        <x:v>ProTek Texturbase White=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/textureline-ProTek-Texturbase-White-SDS.pdf?raw=true|ProTek Texturbase Neutral=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/textureline-ProTek-Texturbase-Neutral-SDS.pdf?raw=true</x:v>
+      </x:c>
+      <x:c r="Z630" t="str">
+        <x:v>ProTek Acrylic Venetian Plaster=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/textureline-ProTek-Acrylic-Venetian-Plaster-System-TDS.pdf?raw=true</x:v>
+      </x:c>
     </x:row>
     <x:row r="631">
       <x:c r="A631" t="str">
@@ -32254,6 +32311,12 @@
       <x:c r="U632" t="str"/>
       <x:c r="V632" t="str"/>
       <x:c r="W632" t="str"/>
+      <x:c r="X632" t="str">
+        <x:v>ProTek Marmorino Classico=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/textureline-ProTek-Marmorino-Classico-SDS.pdf?raw=true</x:v>
+      </x:c>
+      <x:c r="Z632" t="str">
+        <x:v>ProTek Marmorino Classico Venetian Plaster=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/textureline-ProTek-Marmorino-Classico-Venetian-Plaster-TDS.pdf?raw=true</x:v>
+      </x:c>
     </x:row>
     <x:row r="633">
       <x:c r="A633" t="str">

</xml_diff>

<commit_message>
Add Roman and Rosco coating documents 177-184
</commit_message>
<xml_diff>
--- a/products_categories_descriptions_documents_working.xlsx
+++ b/products_categories_descriptions_documents_working.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" r:id="R2972247848a24863"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" r:id="R45149da703e34348"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -32740,6 +32740,12 @@
       <x:c r="U641" t="str"/>
       <x:c r="V641" t="str"/>
       <x:c r="W641" t="str"/>
+      <x:c r="X641" t="str">
+        <x:v>ROMAN PRO-999 Rx-35 Sealer/Primer=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/roman-ROMAN-PRO-999-Rx-35-Sealer-Primer-SDS.pdf?raw=true</x:v>
+      </x:c>
+      <x:c r="Z641" t="str">
+        <x:v>ROMAN PRO-999 Rx-35 Sealer/Primer=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/roman-ROMAN-PRO-999-Rx-35-Sealer-Primer-TDS.pdf?raw=true</x:v>
+      </x:c>
     </x:row>
     <x:row r="642">
       <x:c r="A642" t="str">
@@ -32787,6 +32793,12 @@
       <x:c r="U642" t="str"/>
       <x:c r="V642" t="str"/>
       <x:c r="W642" t="str"/>
+      <x:c r="X642" t="str">
+        <x:v>ROMAN PRO-977 Ultra Prime - Canada English=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/roman-ROMAN-PRO-977-Ultra-Prime-CA-EN-SDS.pdf?raw=true</x:v>
+      </x:c>
+      <x:c r="Z642" t="str">
+        <x:v>ROMAN PRO-977 Ultra Prime=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/roman-ROMAN-PRO-977-Ultra-Prime-TDS.pdf?raw=true</x:v>
+      </x:c>
     </x:row>
     <x:row r="643">
       <x:c r="A643" t="str">
@@ -32928,6 +32940,9 @@
       <x:c r="U645" t="str"/>
       <x:c r="V645" t="str"/>
       <x:c r="W645" t="str"/>
+      <x:c r="X645" t="str">
+        <x:v>Rosco Video Screen Paint RF7900=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/rosco-Rosco-Video-Screen-Paint-RF7900-SDS.pdf?raw=true</x:v>
+      </x:c>
     </x:row>
     <x:row r="646">
       <x:c r="A646" t="str">
@@ -32975,6 +32990,12 @@
       <x:c r="U646" t="str"/>
       <x:c r="V646" t="str"/>
       <x:c r="W646" t="str"/>
+      <x:c r="X646" t="str">
+        <x:v>Rosco Chroma Key Green 5711=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/rosco-Rosco-Chroma-Key-Green-5711-SDS.pdf?raw=true</x:v>
+      </x:c>
+      <x:c r="Z646" t="str">
+        <x:v>Rosco Chroma Key Paint Application Guide=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/rosco-Rosco-Chroma-Key-Paint-Application-Guide-TDS.pdf?raw=true</x:v>
+      </x:c>
     </x:row>
     <x:row r="647">
       <x:c r="A647" t="str">
@@ -33022,6 +33043,12 @@
       <x:c r="U647" t="str"/>
       <x:c r="V647" t="str"/>
       <x:c r="W647" t="str"/>
+      <x:c r="X647" t="str">
+        <x:v>Rosco Chroma Key Blue 5710=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/rosco-Rosco-Chroma-Key-Blue-5710-SDS.pdf?raw=true</x:v>
+      </x:c>
+      <x:c r="Z647" t="str">
+        <x:v>Rosco Chroma Key Paint Application Guide=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/rosco-Rosco-Chroma-Key-Paint-Application-Guide-TDS.pdf?raw=true</x:v>
+      </x:c>
     </x:row>
     <x:row r="648">
       <x:c r="A648" t="str">
@@ -33069,6 +33096,9 @@
       <x:c r="U648" t="str"/>
       <x:c r="V648" t="str"/>
       <x:c r="W648" t="str"/>
+      <x:c r="X648" t="str">
+        <x:v>Rosco TV Paint White 5735=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/rosco-Rosco-TV-Paint-White-5735-SDS.pdf?raw=true</x:v>
+      </x:c>
     </x:row>
     <x:row r="649">
       <x:c r="A649" t="str">
@@ -33116,6 +33146,9 @@
       <x:c r="U649" t="str"/>
       <x:c r="V649" t="str"/>
       <x:c r="W649" t="str"/>
+      <x:c r="X649" t="str">
+        <x:v>Rosco TV Paint Black 5740=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/rosco-Rosco-TV-Paint-Black-5740-SDS.pdf?raw=true</x:v>
+      </x:c>
     </x:row>
     <x:row r="650">
       <x:c r="A650" t="str">
@@ -33163,6 +33196,12 @@
       <x:c r="U650" t="str"/>
       <x:c r="V650" t="str"/>
       <x:c r="W650" t="str"/>
+      <x:c r="X650" t="str">
+        <x:v>Roscoflamex PA Paint Additive=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/rosco-Roscoflamex-PA-Paint-Additive-SDS.pdf?raw=true</x:v>
+      </x:c>
+      <x:c r="Z650" t="str">
+        <x:v>Roscoflamex PA Paint Additive=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/rosco-Roscoflamex-PA-Paint-Additive-Specification-TDS.pdf?raw=true</x:v>
+      </x:c>
     </x:row>
     <x:row r="651">
       <x:c r="A651" t="str">

</xml_diff>

<commit_message>
Add Rust-Oleum coating documents 185-195
</commit_message>
<xml_diff>
--- a/products_categories_descriptions_documents_working.xlsx
+++ b/products_categories_descriptions_documents_working.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" r:id="R45149da703e34348"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" r:id="R69b5880a07344780"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -33445,6 +33445,12 @@
       <x:c r="U655" t="str"/>
       <x:c r="V655" t="str"/>
       <x:c r="W655" t="str"/>
+      <x:c r="X655" t="str">
+        <x:v>SEAL-KRETE Clear-Seal Clear Satin 3.78 L - 604801=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/seal-krete-SEAL-KRETE-Clear-Seal-Satin-604801-SDS.pdf?raw=true</x:v>
+      </x:c>
+      <x:c r="AA655" t="str">
+        <x:v>SEAL-KRETE Clear-Seal SLK-14=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/seal-krete-SEAL-KRETE-Clear-Seal-SLK-14-TDS.pdf?raw=true</x:v>
+      </x:c>
     </x:row>
     <x:row r="656">
       <x:c r="A656" t="str">
@@ -33492,6 +33498,12 @@
       <x:c r="U656" t="str"/>
       <x:c r="V656" t="str"/>
       <x:c r="W656" t="str"/>
+      <x:c r="X656" t="str">
+        <x:v>Rust-Oleum Tub &amp; Tile Refinishing Kit Gloss Coastal Fog - 384166=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/rust-oleum-Rust-Oleum-Tub-Tile-Gloss-Coastal-Fog-384166-SDS.pdf?raw=true</x:v>
+      </x:c>
+      <x:c r="Z656" t="str">
+        <x:v>Rust-Oleum Tub &amp; Tile Refinishing Kit SPC-15 - includes 384166=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/rust-oleum-Rust-Oleum-Tub-Tile-Refinishing-Kit-SPC-15-TDS.pdf?raw=true</x:v>
+      </x:c>
     </x:row>
     <x:row r="657">
       <x:c r="A657" t="str">
@@ -33539,6 +33551,12 @@
       <x:c r="U657" t="str"/>
       <x:c r="V657" t="str"/>
       <x:c r="W657" t="str"/>
+      <x:c r="X657" t="str">
+        <x:v>Rust-Oleum Automotive Self-Etching Primer Grey-Green 340 g - 257736=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/rust-oleum-Rust-Oleum-Automotive-Self-Etching-Primer-257736-SDS.pdf?raw=true</x:v>
+      </x:c>
+      <x:c r="Z657" t="str">
+        <x:v>Rust-Oleum Automotive Self-Etching Primer ATO-151 Canada=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/rust-oleum-Rust-Oleum-Automotive-Self-Etching-Primer-ATO-151-Canada-TDS.pdf?raw=true</x:v>
+      </x:c>
     </x:row>
     <x:row r="658">
       <x:c r="A658" t="str">
@@ -33586,6 +33604,12 @@
       <x:c r="U658" t="str"/>
       <x:c r="V658" t="str"/>
       <x:c r="W658" t="str"/>
+      <x:c r="X658" t="str">
+        <x:v>Rust-Oleum Mirror Effect Silver 170 g - 277903=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/rust-oleum-Rust-Oleum-Mirror-Effect-Silver-277903-SDS.pdf?raw=true</x:v>
+      </x:c>
+      <x:c r="Z658" t="str">
+        <x:v>Rust-Oleum Mirror Effect SPC-36 Canada=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/rust-oleum-Rust-Oleum-Mirror-Effect-SPC-36-Canada-TDS.pdf?raw=true</x:v>
+      </x:c>
     </x:row>
     <x:row r="659">
       <x:c r="A659" t="str">
@@ -33633,6 +33657,12 @@
       <x:c r="U659" t="str"/>
       <x:c r="V659" t="str"/>
       <x:c r="W659" t="str"/>
+      <x:c r="X659" t="str">
+        <x:v>Rust-Oleum Specialty Metallic Gold 312 g - N1910830=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/rust-oleum-Rust-Oleum-Specialty-Metallic-Gold-N1910830-SDS.pdf?raw=true</x:v>
+      </x:c>
+      <x:c r="Z659" t="str">
+        <x:v>Rust-Oleum Specialty Metallic Sprays SPC-13 - includes 1910830=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/rust-oleum-Rust-Oleum-Specialty-Metallic-SPC-13-TDS.pdf?raw=true</x:v>
+      </x:c>
     </x:row>
     <x:row r="660">
       <x:c r="A660" t="str">
@@ -33680,6 +33710,12 @@
       <x:c r="U660" t="str"/>
       <x:c r="V660" t="str"/>
       <x:c r="W660" t="str"/>
+      <x:c r="X660" t="str">
+        <x:v>Rust-Oleum LeakSeal Flexible Rubber Sealant Clear 405 g - 266289=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/rust-oleum-Rust-Oleum-LeakSeal-Clear-266289-SDS.pdf?raw=true</x:v>
+      </x:c>
+      <x:c r="Z660" t="str">
+        <x:v>Rust-Oleum LeakSeal Flexible Rubber Coating SRT-17=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/rust-oleum-Rust-Oleum-LeakSeal-Flexible-Rubber-Coating-SRT-17-TDS.pdf?raw=true</x:v>
+      </x:c>
     </x:row>
     <x:row r="661">
       <x:c r="A661" t="str">
@@ -33727,6 +33763,12 @@
       <x:c r="U661" t="str"/>
       <x:c r="V661" t="str"/>
       <x:c r="W661" t="str"/>
+      <x:c r="X661" t="str">
+        <x:v>Rust-Oleum LeakSeal Flexible Rubber Sealant Black 405 g - 266288=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/rust-oleum-Rust-Oleum-LeakSeal-Black-266288-SDS.pdf?raw=true</x:v>
+      </x:c>
+      <x:c r="Z661" t="str">
+        <x:v>Rust-Oleum LeakSeal Flexible Rubber Coating SRT-17=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/rust-oleum-Rust-Oleum-LeakSeal-Flexible-Rubber-Coating-SRT-17-TDS.pdf?raw=true</x:v>
+      </x:c>
     </x:row>
     <x:row r="662">
       <x:c r="A662" t="str">
@@ -33774,6 +33816,12 @@
       <x:c r="U662" t="str"/>
       <x:c r="V662" t="str"/>
       <x:c r="W662" t="str"/>
+      <x:c r="X662" t="str">
+        <x:v>Rust-Oleum Appliance Epoxy Gloss White 340 g - N7881830=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/rust-oleum-Rust-Oleum-Appliance-Epoxy-Gloss-White-N7881830-SDS.pdf?raw=true</x:v>
+      </x:c>
+      <x:c r="Z662" t="str">
+        <x:v>Rust-Oleum Specialty Appliance Epoxy Sprays SPC-01 - includes 7881830=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/rust-oleum-Rust-Oleum-Appliance-Epoxy-Sprays-SPC-01-TDS.pdf?raw=true</x:v>
+      </x:c>
     </x:row>
     <x:row r="663">
       <x:c r="A663" t="str">
@@ -33829,6 +33877,9 @@
       <x:c r="U663" t="str"/>
       <x:c r="V663" t="str"/>
       <x:c r="W663" t="str"/>
+      <x:c r="X663" t="str">
+        <x:v>Rust-Oleum Painter's Touch Multi-Purpose Latex Flat Black 946 mL - 254935=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/rust-oleum-Rust-Oleum-Painters-Touch-Latex-Flat-Black-254935-SDS.pdf?raw=true</x:v>
+      </x:c>
     </x:row>
     <x:row r="664">
       <x:c r="A664" t="str">
@@ -33876,6 +33927,9 @@
       <x:c r="U664" t="str"/>
       <x:c r="V664" t="str"/>
       <x:c r="W664" t="str"/>
+      <x:c r="X664" t="str">
+        <x:v>TREMCLAD Rust Primer Spray Red Oxide 340 g - 274102522=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/tremclad-TREMCLAD-Rust-Primer-Spray-Red-Oxide-274102522-SDS.pdf?raw=true</x:v>
+      </x:c>
     </x:row>
     <x:row r="665">
       <x:c r="A665" t="str">
@@ -33923,6 +33977,12 @@
       <x:c r="U665" t="str"/>
       <x:c r="V665" t="str"/>
       <x:c r="W665" t="str"/>
+      <x:c r="X665" t="str">
+        <x:v>TREMCLAD Rust Paint Aerosol Gloss Recreational White 340 g - 27032B522=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/tremclad-TREMCLAD-Rust-Paint-Aerosol-Recreational-White-27032B522-SDS.pdf?raw=true</x:v>
+      </x:c>
+      <x:c r="Z665" t="str">
+        <x:v>TREMCLAD Rust Paint Aerosol TRM-02 Canada=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/tremclad-TRM-02-Tremclad-Rust-Paint-Aerosol-TDS-Canada.pdf?raw=true</x:v>
+      </x:c>
     </x:row>
     <x:row r="666">
       <x:c r="A666" t="str">

</xml_diff>

<commit_message>
Add Ready Seal and SamaN coating documents 196-202
</commit_message>
<xml_diff>
--- a/products_categories_descriptions_documents_working.xlsx
+++ b/products_categories_descriptions_documents_working.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" r:id="R69b5880a07344780"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" r:id="Rb8376f3a58624cd2"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -34171,6 +34171,12 @@
       <x:c r="U669" t="str"/>
       <x:c r="V669" t="str"/>
       <x:c r="W669" t="str"/>
+      <x:c r="X669" t="str">
+        <x:v>Ready Seal Exterior Wood Stain Natural No. 105 - Canada=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/ready-seal-Ready-Seal-Exterior-Wood-Stain-Natural-105-Canada-SDS.pdf?raw=true</x:v>
+      </x:c>
+      <x:c r="Z669" t="str">
+        <x:v>Ready Seal Exterior Wood Stain and Sealer=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/ready-seal-Ready-Seal-Exterior-Wood-Stain-Sealer-TDS.pdf?raw=true</x:v>
+      </x:c>
     </x:row>
     <x:row r="670">
       <x:c r="A670" t="str">
@@ -34218,6 +34224,9 @@
       <x:c r="U670" t="str"/>
       <x:c r="V670" t="str"/>
       <x:c r="W670" t="str"/>
+      <x:c r="X670" t="str">
+        <x:v>SamaN Waterbased Exterior Clear Coat Flat - SAM-805=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/saman-SamaN-Waterbased-Exterior-Clear-Coat-SAM-805-SDS.pdf?raw=true</x:v>
+      </x:c>
     </x:row>
     <x:row r="671">
       <x:c r="A671" t="str">
@@ -34265,6 +34274,12 @@
       <x:c r="U671" t="str"/>
       <x:c r="V671" t="str"/>
       <x:c r="W671" t="str"/>
+      <x:c r="X671" t="str">
+        <x:v>SamaN Water-Based Wood Stain Whole Wheat 010=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/saman-SamaN-Water-Based-Wood-Stain-TEW-SDS.pdf?raw=true</x:v>
+      </x:c>
+      <x:c r="Z671" t="str">
+        <x:v>SamaN Water-Based Wood Stain TEW=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/saman-SamaN-Water-Based-Wood-Stain-TEW-TDS.pdf?raw=true</x:v>
+      </x:c>
     </x:row>
     <x:row r="672">
       <x:c r="A672" t="str">
@@ -34312,6 +34327,9 @@
       <x:c r="U672" t="str"/>
       <x:c r="V672" t="str"/>
       <x:c r="W672" t="str"/>
+      <x:c r="X672" t="str">
+        <x:v>SamaN Waterbased Glaze Regular - CG-100=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/saman-SamaN-Waterbased-Glaze-CG-100-SDS.pdf?raw=true</x:v>
+      </x:c>
     </x:row>
     <x:row r="673">
       <x:c r="A673" t="str">
@@ -34359,6 +34377,12 @@
       <x:c r="U673" t="str"/>
       <x:c r="V673" t="str"/>
       <x:c r="W673" t="str"/>
+      <x:c r="X673" t="str">
+        <x:v>SamaN Legend Tung Oil Natural - TOH-000=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/saman-SamaN-Legend-Tung-Oil-Natural-TOH-000-SDS.pdf?raw=true</x:v>
+      </x:c>
+      <x:c r="Z673" t="str">
+        <x:v>SamaN Legend Tung Oil TOH-000 and TOH-401 to TOH-409=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/saman-SamaN-Legend-Tung-Oil-TOH-TDS.pdf?raw=true</x:v>
+      </x:c>
     </x:row>
     <x:row r="674">
       <x:c r="A674" t="str">
@@ -34406,6 +34430,9 @@
       <x:c r="U674" t="str"/>
       <x:c r="V674" t="str"/>
       <x:c r="W674" t="str"/>
+      <x:c r="X674" t="str">
+        <x:v>SamaN EPOX-Y Counter Bar Table Epoxy Part A Resin - EPO-100A-500=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/saman-SamaN-EPOX-Y-Tabletop-Epoxy-EPO-100A-500-EN-SDS.pdf?raw=true|SamaN EPOX-Y Counter Bar Table Epoxy Part B Hardener - EPO-100B-500=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/saman-SamaN-EPOX-Y-Tabletop-Epoxy-EPO-100B-500-EN-SDS.pdf?raw=true</x:v>
+      </x:c>
     </x:row>
     <x:row r="675">
       <x:c r="A675" t="str">
@@ -34547,6 +34574,9 @@
       <x:c r="U677" t="str"/>
       <x:c r="V677" t="str"/>
       <x:c r="W677" t="str"/>
+      <x:c r="X677" t="str">
+        <x:v>SamaN Natural Beeswax Wood Finish and Conditioner - BWA-000=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/saman-SamaN-Natural-Beeswax-BWA-000-SDS.pdf?raw=true</x:v>
+      </x:c>
     </x:row>
     <x:row r="678">
       <x:c r="A678" t="str">

</xml_diff>

<commit_message>
Add Seal King and ALLPRO coating documents 203-207
</commit_message>
<xml_diff>
--- a/products_categories_descriptions_documents_working.xlsx
+++ b/products_categories_descriptions_documents_working.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" r:id="Rb8376f3a58624cd2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" r:id="R8a4e0a81b07d4941"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -34812,6 +34812,12 @@
       <x:c r="U682" t="str"/>
       <x:c r="V682" t="str"/>
       <x:c r="W682" t="str"/>
+      <x:c r="X682" t="str">
+        <x:v>Seal King Paving Stone Sealer Semi Gloss=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/seal-king-Seal-King-Paving-Stone-Sealer-Semi-Gloss-SDS.pdf?raw=true</x:v>
+      </x:c>
+      <x:c r="Z682" t="str">
+        <x:v>Seal King Paving Stone Sealer - includes Semi Gloss=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/seal-king-Seal-King-Paving-Stone-Sealer-TDS.pdf?raw=true</x:v>
+      </x:c>
     </x:row>
     <x:row r="683">
       <x:c r="A683" t="str">
@@ -34906,6 +34912,12 @@
       <x:c r="U684" t="str"/>
       <x:c r="V684" t="str"/>
       <x:c r="W684" t="str"/>
+      <x:c r="X684" t="str">
+        <x:v>Seal King Natural Stone Sealer Natural Look - SK/NSSN=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/seal-king-Seal-King-Natural-Stone-Sealer-Natural-Look-SDS.pdf?raw=true</x:v>
+      </x:c>
+      <x:c r="Z684" t="str">
+        <x:v>Seal King Natural Stone Sealer - Natural Look and Colour Enhancer - French=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/seal-king-Seal-King-Natural-Stone-Sealer-TDS.pdf?raw=true</x:v>
+      </x:c>
     </x:row>
     <x:row r="685">
       <x:c r="A685" t="str">
@@ -34953,6 +34965,12 @@
       <x:c r="U685" t="str"/>
       <x:c r="V685" t="str"/>
       <x:c r="W685" t="str"/>
+      <x:c r="X685" t="str">
+        <x:v>Seal King Natural Stone Sealer Colour Enhancer - SK/NSSCE=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/seal-king-Seal-King-Natural-Stone-Sealer-Colour-Enhancer-SDS.pdf?raw=true</x:v>
+      </x:c>
+      <x:c r="Z685" t="str">
+        <x:v>Seal King Natural Stone Sealer - Natural Look and Colour Enhancer - French=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/seal-king-Seal-King-Natural-Stone-Sealer-TDS.pdf?raw=true</x:v>
+      </x:c>
     </x:row>
     <x:row r="686">
       <x:c r="A686" t="str">
@@ -35141,6 +35159,12 @@
       <x:c r="U689" t="str"/>
       <x:c r="V689" t="str"/>
       <x:c r="W689" t="str"/>
+      <x:c r="X689" t="str">
+        <x:v>Seal King Basement Floor Sealer Clear - SK/BFS=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/seal-king-Seal-King-Basement-Floor-Sealer-Clear-SDS.pdf?raw=true</x:v>
+      </x:c>
+      <x:c r="Z689" t="str">
+        <x:v>Seal King Basement Floor Sealer Clear=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/seal-king-Seal-King-Basement-Floor-Sealer-Clear-TDS.pdf?raw=true</x:v>
+      </x:c>
     </x:row>
     <x:row r="690">
       <x:c r="A690" t="str">
@@ -35188,6 +35212,12 @@
       <x:c r="U690" t="str"/>
       <x:c r="V690" t="str"/>
       <x:c r="W690" t="str"/>
+      <x:c r="X690" t="str">
+        <x:v>ALLPRO Spray Enamel Fire Engine Red - 11051=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/allpro-ALLPRO-Spray-Enamel-Fire-Engine-Red-11051-SDS.pdf?raw=true</x:v>
+      </x:c>
+      <x:c r="Z690" t="str">
+        <x:v>ALLPRO Spray Enamel 11050-11068 - includes 11051 Fire Engine Red=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/allpro-ALLPRO-Spray-Enamel-11050-11068-TDS.pdf?raw=true</x:v>
+      </x:c>
     </x:row>
     <x:row r="691">
       <x:c r="A691" t="str">

</xml_diff>

<commit_message>
Add Sikkens coating documents 208-212
</commit_message>
<xml_diff>
--- a/products_categories_descriptions_documents_working.xlsx
+++ b/products_categories_descriptions_documents_working.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" r:id="R8a4e0a81b07d4941"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" r:id="Rdf21ce826a9e4067"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -35594,6 +35594,12 @@
       <x:c r="U698" t="str"/>
       <x:c r="V698" t="str"/>
       <x:c r="W698" t="str"/>
+      <x:c r="X698" t="str">
+        <x:v>PPG ProLuxe SRD RE Natural Oak 005 - SIK250-005/01=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/sikkens-PPG-ProLuxe-SRD-RE-Natural-Oak-005-SDS.pdf?raw=true</x:v>
+      </x:c>
+      <x:c r="Z698" t="str">
+        <x:v>PPG ProLuxe SRD RE Natural Oak 005 - SIK250-005/01=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/sikkens-PPG-ProLuxe-SRD-RE-Natural-Oak-005-TDS.pdf?raw=true</x:v>
+      </x:c>
     </x:row>
     <x:row r="699">
       <x:c r="A699" t="str">
@@ -35641,6 +35647,12 @@
       <x:c r="U699" t="str"/>
       <x:c r="V699" t="str"/>
       <x:c r="W699" t="str"/>
+      <x:c r="X699" t="str">
+        <x:v>PPG ProLuxe Premium Deck Cedar 077 - SIK44077/01=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/sikkens-PPG-ProLuxe-Premium-Deck-Cedar-077-SDS.pdf?raw=true</x:v>
+      </x:c>
+      <x:c r="Z699" t="str">
+        <x:v>PPG ProLuxe Premium Deck Cedar 077 - SIK44077/01=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/sikkens-PPG-ProLuxe-Premium-Deck-Cedar-077-TDS.pdf?raw=true</x:v>
+      </x:c>
     </x:row>
     <x:row r="700">
       <x:c r="A700" t="str">
@@ -35688,6 +35700,12 @@
       <x:c r="U700" t="str"/>
       <x:c r="V700" t="str"/>
       <x:c r="W700" t="str"/>
+      <x:c r="X700" t="str">
+        <x:v>PPG ProLuxe Door &amp; Window Satin Colorless - SIK48003/01=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/sikkens-PPG-ProLuxe-Door-Window-Satin-Colorless-SDS.pdf?raw=true</x:v>
+      </x:c>
+      <x:c r="Z700" t="str">
+        <x:v>PPG ProLuxe Door &amp; Window Satin Colorless - SIK48003/01=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/sikkens-PPG-ProLuxe-Door-Window-Satin-Colorless-TDS.pdf?raw=true</x:v>
+      </x:c>
     </x:row>
     <x:row r="701">
       <x:c r="A701" t="str">
@@ -35735,6 +35753,12 @@
       <x:c r="U701" t="str"/>
       <x:c r="V701" t="str"/>
       <x:c r="W701" t="str"/>
+      <x:c r="X701" t="str">
+        <x:v>PPG ProLuxe 23 Top Coat RE Natural Oak 005 - SIK43005/01=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/sikkens-PPG-ProLuxe-23-Top-Coat-RE-Natural-Oak-005-SDS.pdf?raw=true</x:v>
+      </x:c>
+      <x:c r="Z701" t="str">
+        <x:v>PPG ProLuxe 23 Top Coat RE Natural Oak 005 - SIK43005/01=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/sikkens-PPG-ProLuxe-23-Top-Coat-RE-Natural-Oak-005-TDS.pdf?raw=true</x:v>
+      </x:c>
     </x:row>
     <x:row r="702">
       <x:c r="A702" t="str">
@@ -35782,6 +35806,12 @@
       <x:c r="U702" t="str"/>
       <x:c r="V702" t="str"/>
       <x:c r="W702" t="str"/>
+      <x:c r="X702" t="str">
+        <x:v>PPG ProLuxe 1 Primary Coat RE Natural Oak 005 - SIK41005/01=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/sikkens-PPG-ProLuxe-1-Primary-Coat-RE-Natural-Oak-005-SDS.pdf?raw=true</x:v>
+      </x:c>
+      <x:c r="Z702" t="str">
+        <x:v>PPG ProLuxe 1 Primary Coat RE Natural Oak 005 - SIK41005/01=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/sikkens-PPG-ProLuxe-1-Primary-Coat-RE-Natural-Oak-005-TDS.pdf?raw=true</x:v>
+      </x:c>
     </x:row>
     <x:row r="703">
       <x:c r="A703" t="str">

</xml_diff>

<commit_message>
Add Simiron coating documents 213-215
</commit_message>
<xml_diff>
--- a/products_categories_descriptions_documents_working.xlsx
+++ b/products_categories_descriptions_documents_working.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" r:id="Rdf21ce826a9e4067"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" r:id="R8074d9ac710f4333"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -35859,6 +35859,12 @@
       <x:c r="U703" t="str"/>
       <x:c r="V703" t="str"/>
       <x:c r="W703" t="str"/>
+      <x:c r="X703" t="str">
+        <x:v>Simiron Smark Fill Me Base component=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/simiron-Simiron-Smark-Fill-Me-Base-SDS.pdf?raw=true|Simiron Smark Pour Me Activator component=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/simiron-Simiron-Smark-Pour-Me-Activator-SDS.pdf?raw=true</x:v>
+      </x:c>
+      <x:c r="Z703" t="str">
+        <x:v>Simiron Smark Clear Dry Erase Paint - includes 200 sq. ft. kit 40002930=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/simiron-Simiron-Smark-Clear-Dry-Erase-Paint-TDS.pdf?raw=true</x:v>
+      </x:c>
     </x:row>
     <x:row r="704">
       <x:c r="A704" t="str">

</xml_diff>

<commit_message>
Add Brodi Renner and Watco documents 216-218
</commit_message>
<xml_diff>
--- a/products_categories_descriptions_documents_working.xlsx
+++ b/products_categories_descriptions_documents_working.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" r:id="R8074d9ac710f4333"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" r:id="Rab2b537c5ddc499f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -38693,6 +38693,9 @@
       <x:c r="U763" t="str"/>
       <x:c r="V763" t="str"/>
       <x:c r="W763" t="str"/>
+      <x:c r="X763" t="str">
+        <x:v>Brodi Renew Acoustical Ceiling Tile Restorer=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/value-chem-Brodi-Renew-Acoustical-Ceiling-Tile-Restorer-SDS.pdf?raw=true</x:v>
+      </x:c>
     </x:row>
     <x:row r="764">
       <x:c r="A764" t="str">
@@ -38928,6 +38931,9 @@
       <x:c r="U768" t="str"/>
       <x:c r="V768" t="str"/>
       <x:c r="W768" t="str"/>
+      <x:c r="AA768" t="str">
+        <x:v>Renner Larice exterior varnish 30 sheen - YO30.1061.609AUS=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/renner-Renner-Larice-YO30-1061-609AUS-TDS.pdf?raw=true</x:v>
+      </x:c>
     </x:row>
     <x:row r="769">
       <x:c r="A769" t="str">
@@ -39022,6 +39028,12 @@
       <x:c r="U770" t="str"/>
       <x:c r="V770" t="str"/>
       <x:c r="W770" t="str"/>
+      <x:c r="X770" t="str">
+        <x:v>Watco Danish Oil Dark Walnut - Y65841H=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/watco-Watco-Danish-Oil-Dark-Walnut-Y65841H-SDS.pdf?raw=true</x:v>
+      </x:c>
+      <x:c r="Z770" t="str">
+        <x:v>Watco Danish Oil - includes Dark Walnut=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/watco-Watco-Danish-Oil-Dark-Walnut-TDS.pdf?raw=true</x:v>
+      </x:c>
     </x:row>
     <x:row r="771">
       <x:c r="A771" t="str">

</xml_diff>

<commit_message>
Add XIM Howard and Zinsser documents 219-221
</commit_message>
<xml_diff>
--- a/products_categories_descriptions_documents_working.xlsx
+++ b/products_categories_descriptions_documents_working.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" r:id="Rab2b537c5ddc499f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" r:id="R82b5d44c2ebf4af6"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -39880,6 +39880,12 @@
       <x:c r="U788" t="str"/>
       <x:c r="V788" t="str"/>
       <x:c r="W788" t="str"/>
+      <x:c r="X788" t="str">
+        <x:v>X-I-M UMA Advanced Technology White 1-Gallon - 11051=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/xim-XIM-UMA-Advanced-Technology-White-11051-SDS.pdf?raw=true</x:v>
+      </x:c>
+      <x:c r="Z788" t="str">
+        <x:v>X-I-M UMA Advanced Technology Primer Sealer Bonder White - includes 1-Gallon 11051=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/xim-XIM-UMA-Advanced-Technology-White-TDS.pdf?raw=true</x:v>
+      </x:c>
     </x:row>
     <x:row r="789">
       <x:c r="A789" t="str">
@@ -39927,6 +39933,12 @@
       <x:c r="U789" t="str"/>
       <x:c r="V789" t="str"/>
       <x:c r="W789" t="str"/>
+      <x:c r="X789" t="str">
+        <x:v>Howard Restor-A-Finish - includes Walnut=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/howard-Howard-Restor-A-Finish-Walnut-SDS.pdf?raw=true</x:v>
+      </x:c>
+      <x:c r="Z789" t="str">
+        <x:v>Howard Restor-A-Finish Fact Sheet - includes Walnut=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/howard-Howard-Restor-A-Finish-Walnut-Fact-Sheet-TDS.pdf?raw=true</x:v>
+      </x:c>
     </x:row>
     <x:row r="790">
       <x:c r="A790" t="str">
@@ -40021,6 +40033,12 @@
       <x:c r="U791" t="str"/>
       <x:c r="V791" t="str"/>
       <x:c r="W791" t="str"/>
+      <x:c r="X791" t="str">
+        <x:v>Zinsser Odor Killing Primer Clear 1-Gallon - 305928=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/zinsser-Zinsser-Odor-Killing-Primer-305928-SDS.pdf?raw=true</x:v>
+      </x:c>
+      <x:c r="Z791" t="str">
+        <x:v>Zinsser Odor Killing Primer - includes 1-Gallon 305928=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/zinsser-Zinsser-Odor-Killing-Primer-TDS.pdf?raw=true</x:v>
+      </x:c>
     </x:row>
     <x:row r="792">
       <x:c r="A792" t="str">

</xml_diff>

<commit_message>
Add final Zinsser coating documents 222-225
</commit_message>
<xml_diff>
--- a/products_categories_descriptions_documents_working.xlsx
+++ b/products_categories_descriptions_documents_working.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" r:id="R82b5d44c2ebf4af6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" r:id="R55e662c157ee4632"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -40086,6 +40086,12 @@
       <x:c r="U792" t="str"/>
       <x:c r="V792" t="str"/>
       <x:c r="W792" t="str"/>
+      <x:c r="X792" t="str">
+        <x:v>Zinsser Covers Up Ceiling Paint &amp; Primer White 454 g Aerosol - Z03696=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/zinsser-Zinsser-Covers-Up-Z03696-SDS.pdf?raw=true</x:v>
+      </x:c>
+      <x:c r="Z792" t="str">
+        <x:v>Zinsser Covers Up Ceiling Paint &amp; Primer - includes Z03696=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/zinsser-Zinsser-Covers-Up-Ceiling-Paint-Primer-TDS.pdf?raw=true</x:v>
+      </x:c>
     </x:row>
     <x:row r="793">
       <x:c r="A793" t="str">
@@ -40149,6 +40155,12 @@
       </x:c>
       <x:c r="V793" t="str"/>
       <x:c r="W793" t="str"/>
+      <x:c r="X793" t="str">
+        <x:v>Zinsser Bulls Eye Shellac Amber 473 mL - Z00718=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/zinsser-Zinsser-Bulls-Eye-Shellac-Amber-Z00718-SDS.pdf?raw=true</x:v>
+      </x:c>
+      <x:c r="Z793" t="str">
+        <x:v>Zinsser Bulls Eye Shellac - Amber and Clear brush formats=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/zinsser-Zinsser-Bulls-Eye-Shellac-TDS.pdf?raw=true</x:v>
+      </x:c>
     </x:row>
     <x:row r="794">
       <x:c r="A794" t="str">
@@ -40243,6 +40255,12 @@
       <x:c r="U795" t="str"/>
       <x:c r="V795" t="str"/>
       <x:c r="W795" t="str"/>
+      <x:c r="X795" t="str">
+        <x:v>Zinsser Shieldz Universal Wallcovering Primer White 1-Gallon - 2501=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/zinsser-Zinsser-Shieldz-Universal-Wallcovering-Primer-2501-SDS.pdf?raw=true</x:v>
+      </x:c>
+      <x:c r="Z795" t="str">
+        <x:v>Zinsser Shieldz Universal Wallcovering Primer - SHZ-02=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/zinsser-Zinsser-Shieldz-Universal-Wallcovering-Primer-TDS.pdf?raw=true</x:v>
+      </x:c>
     </x:row>
     <x:row r="796">
       <x:c r="A796" t="str">
@@ -40290,6 +40308,12 @@
       <x:c r="U796" t="str"/>
       <x:c r="V796" t="str"/>
       <x:c r="W796" t="str"/>
+      <x:c r="X796" t="str">
+        <x:v>Zinsser Peel Stop Plus High Build Binding Primer 946 mL - 266847=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/zinsser-Zinsser-Peel-Stop-Plus-266847-SDS.pdf?raw=true</x:v>
+      </x:c>
+      <x:c r="Z796" t="str">
+        <x:v>Zinsser Peel Stop Plus High Build Binding Primer - includes 946 mL 266847=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/zinsser-Zinsser-Peel-Stop-Plus-High-Build-Binding-Primer-TDS.pdf?raw=true</x:v>
+      </x:c>
     </x:row>
     <x:row r="797">
       <x:c r="A797" t="str">

</xml_diff>

<commit_message>
Add missed coating documents 226-229
</commit_message>
<xml_diff>
--- a/products_categories_descriptions_documents_working.xlsx
+++ b/products_categories_descriptions_documents_working.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" r:id="R55e662c157ee4632"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" r:id="Ree96f10bc97749b4"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -22954,6 +22954,12 @@
       <x:c r="U441" t="str"/>
       <x:c r="V441" t="str"/>
       <x:c r="W441" t="str"/>
+      <x:c r="X441" t="str">
+        <x:v>Flame Control No. 141 High Gloss polyurethane varnish=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/flame-control-Flame-Control-No-141-High-Gloss-SDS.pdf?raw=true</x:v>
+      </x:c>
+      <x:c r="Z441" t="str">
+        <x:v>Flame Control No. 141 polyurethane varnish - Low, Semi and High Gloss=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/flame-control-Flame-Control-No-141-Varnish-TDS.pdf?raw=true</x:v>
+      </x:c>
     </x:row>
     <x:row r="442">
       <x:c r="A442" t="str">
@@ -23142,6 +23148,12 @@
       <x:c r="U445" t="str"/>
       <x:c r="V445" t="str"/>
       <x:c r="W445" t="str"/>
+      <x:c r="X445" t="str">
+        <x:v>Black Jack Drive-Kote 500 Blacktop Driveway Sealer - 6452-9-30=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/gh-international-Black-Jack-Drive-Kote-500-6452-SDS.pdf?raw=true</x:v>
+      </x:c>
+      <x:c r="Z445" t="str">
+        <x:v>Black Jack Drive-Kote 500 Blacktop Driveway Sealer - 6452=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/gh-international-Black-Jack-Drive-Kote-500-6452-TDS.pdf?raw=true</x:v>
+      </x:c>
     </x:row>
     <x:row r="446">
       <x:c r="A446" t="str">
@@ -25030,6 +25042,9 @@
       <x:c r="U485" t="str"/>
       <x:c r="V485" t="str"/>
       <x:c r="W485" t="str"/>
+      <x:c r="X485" t="str">
+        <x:v>Krylon Metallic Paint Chrome Aluminum - K01404777 / UPC 724504071976=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/krylon-Krylon-Metallic-Chrome-Aluminum-K01404777-SDS.pdf?raw=true</x:v>
+      </x:c>
     </x:row>
     <x:row r="486">
       <x:c r="A486" t="str">
@@ -27375,6 +27390,12 @@
       <x:c r="U531" t="str"/>
       <x:c r="V531" t="str"/>
       <x:c r="W531" t="str"/>
+      <x:c r="X531" t="str">
+        <x:v>Minwax Antique Oil Finish Natural 1 Quart - UPC 027426670006=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/SDS/minwax-Minwax-Antique-Oil-Finish-027426670006-SDS.pdf?raw=true</x:v>
+      </x:c>
+      <x:c r="Z531" t="str">
+        <x:v>Minwax Antique Oil Finish Natural 1 Quart - UPC 027426670006=https://raw.githubusercontent.com/kinggoff/NewSteelesImages/main/PDFs/TDS/minwax-Minwax-Antique-Oil-Finish-027426670006-TDS.pdf?raw=true</x:v>
+      </x:c>
     </x:row>
     <x:row r="532">
       <x:c r="A532" t="str">

</xml_diff>